<commit_message>
Mise à jour automatique 2026-09-13 18:08:29
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,14 +424,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SOKO</t>
+          <t>TOUMODI_RAMBO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IM091</t>
+          <t>ET811</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SOKO</t>
+          <t>TOUMODI_RAMBO</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-11 15:37:27</t>
+          <t>2026-09-13 08:02:57</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-11 15:37:27</t>
+          <t>2026-09-13 08:02:57</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>TOUMODI_RAMBO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>ET811</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>TOUMODI_RAMBO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-11 10:43:57</t>
+          <t>2026-09-13 10:19:56</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-11 10:43:57</t>
+          <t>2026-09-13 10:19:56</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=98/208, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,34 +645,34 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-11 14:42:25</t>
+          <t>2026-09-13 10:55:19</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-11 14:42:25</t>
+          <t>2026-09-13 10:55:19</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -712,24 +712,24 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BAGOLIEOUA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC978</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BAGOLEHOUA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:16:38</t>
+          <t>2026-09-13 13:00:15</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:16:38</t>
+          <t>2026-09-13 13:00:15</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -779,34 +779,34 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-11 15:47:00</t>
+          <t>2026-09-13 13:33:42</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-11 15:47:00</t>
+          <t>2026-09-13 13:33:42</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SOKO</t>
+          <t>TOUMODI_RAMBO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>IM091</t>
+          <t>ET811</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SOKO</t>
+          <t>TOUMODI_RAMBO</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-11 15:56:30</t>
+          <t>2026-09-13 13:37:12</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-11 15:56:30</t>
+          <t>2026-09-13 13:37:12</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=98/208, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,39 +913,39 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-11 10:16:06</t>
+          <t>2026-09-13 14:21:56</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-11 10:16:06</t>
+          <t>2026-09-13 14:21:56</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,49 +970,49 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DABOU_SODECI</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC932</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC932_W</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-11 14:27:25</t>
+          <t>2026-09-13 14:43:59</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-11 14:27:25</t>
+          <t>2026-09-13 14:43:59</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,49 +1037,49 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2577806954</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-13 15:19:39</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-13 15:19:39</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,34 +1104,34 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>YOP_PORT-BOUET2_SIDOCO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>ET991</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_ET991_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,39 +1181,39 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-13 09:03:50</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-13 09:03:50</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-01 23:38:09</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-09 13:01:43</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2572853428</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-11 07:31:00</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-10 13:59:35</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,39 +1449,39 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TERMINAL_2</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ET903</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_ET903_WL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Indoor RAP Temperature Exceptional</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-11 15:59:21</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-11 15:59:21</t>
+          <t>2026-09-12 10:49:55</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET903_WL,ManagedElement=BB_ET903_WL,Equipment=1,FieldReplaceableUnit=RD-1-3 2576221744</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,24 +1516,24 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-10 13:59:35</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,54 +1583,54 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>ABOISSO_MUNICIPALITE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET545</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>Microwave</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>ET545-ML6691</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temperature</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-13 14:34:55</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-13 15:06:47</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=MINILINK,MeContext=ET545-ML6691,ManagedElement=ET545-ML6691,NPU_1003=1/4 2578227022</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1650,39 +1650,39 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>TERMINAL_2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET903</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_ET903_WL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Indoor RAP Temperature Exceptional</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1692,12 +1692,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-13 15:52:28</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-13 15:52:28</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET903_WL,ManagedElement=BB_ET903_WL,Equipment=1,FieldReplaceableUnit=RD-1-3 2576221744</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -1729,12 +1729,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1759,12 +1759,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -1796,12 +1796,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1826,12 +1826,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1851,24 +1851,24 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1893,12 +1893,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1918,57 +1918,54 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>245</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1978,67 +1975,64 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2048,53 +2042,50 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>23</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2103,12 +2094,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2118,67 +2109,64 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>KOUN_ABRONZO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC281</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC281_W</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-11 12:59:36</t>
+          <t>2026-09-13 09:19:55</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-11 12:59:36</t>
+          <t>2026-09-13 11:52:44</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2188,17 +2176,17 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2578506393</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -2210,12 +2198,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2225,7 +2213,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2234,21 +2222,21 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>20</v>
+        <v>245</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-11 15:03:38</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-11 15:03:38</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2246,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=351, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,40 +2256,43 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>31</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -2310,12 +2301,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,64 +2316,67 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>23</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-10 12:25:05</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-10 12:25:05</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,50 +2386,53 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>250</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -2444,12 +2441,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,34 +2456,34 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2496,12 +2493,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2511,12 +2508,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2523,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,24 +2533,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,7 +2560,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2578,12 +2575,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2590,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,24 +2600,24 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NASSIAN</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC546</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,7 +2627,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC546</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2645,12 +2642,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-11 14:53:13</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-11 15:45:01</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2657,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC546,ManagedElement=1,TransportNetwork=1,Synchronization=1 2577557385</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,24 +2667,24 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>FLAKIEDOUGOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC764</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2697,7 +2694,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC764</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2709,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-11 14:53:13</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-11 15:44:59</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2724,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC764,ManagedElement=1,TransportNetwork=1,Synchronization=1 2577557369</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,24 +2734,24 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2764,7 +2761,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2779,12 +2776,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-11 15:14:04</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-11 15:14:04</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2791,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,7 +2801,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -2846,12 +2843,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-11 15:29:21</t>
+          <t>2026-09-13 15:28:11</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-11 15:29:21</t>
+          <t>2026-09-13 15:28:11</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2871,7 +2868,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -2883,22 +2880,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NONOUAN</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC760</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>LAC760</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2913,12 +2910,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-11 15:45:25</t>
+          <t>2026-09-13 15:38:16</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-11 15:45:25</t>
+          <t>2026-09-13 15:38:16</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2928,7 +2925,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576389479</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2938,7 +2935,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -2950,12 +2947,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DAKPADOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AC767</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2965,7 +2962,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>WAC767</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2980,12 +2977,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-11 15:47:25</t>
+          <t>2026-09-13 15:41:38</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-11 15:47:25</t>
+          <t>2026-09-13 15:41:38</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2995,7 +2992,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3005,7 +3002,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -3017,12 +3014,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SASSANDRA_PHARE</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET371</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3032,7 +3029,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>WET371</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3047,12 +3044,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-11 15:47:41</t>
+          <t>2026-09-13 15:46:45</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-11 15:47:41</t>
+          <t>2026-09-13 15:46:45</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3062,7 +3059,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET371,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576049571</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3072,24 +3069,24 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ADEBEM</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ET287</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3099,7 +3096,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>WET287</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3114,12 +3111,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-11 15:48:50</t>
+          <t>2026-09-13 15:52:02</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-11 15:48:50</t>
+          <t>2026-09-13 15:52:02</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3129,7 +3126,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET287,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576087241</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3139,54 +3136,54 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>GESTOCI</t>
+          <t>KOTIESSOU</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC094</t>
+          <t>AC763</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>IP</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>AC094PER6273_01</t>
+          <t>AC763-OSmon</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Transceiver Temperature High Warning</t>
+          <t>Temperature is near limits</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-11 10:31:37</t>
+          <t>1970-01-04 21:21:22</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-11 10:46:22</t>
+          <t>1970-01-04 21:22:38</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3196,7 +3193,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=ROUTER,MeContext=AC094PER6273_01,ManagedElement=1,interfaces=1,interface=2/1 2576388604</t>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2578639730</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3206,57 +3203,54 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>KOTIESSOU</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC763</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>AC763-OSmon</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>1.6</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>1970-01-04 21:22:38</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>1970-01-04 21:22:38</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3266,7 +3260,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2578630038</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3276,24 +3270,24 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3303,7 +3297,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3312,7 +3306,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -3321,12 +3315,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3336,7 +3330,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3346,24 +3340,24 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WILLY_CERES_NORD</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ET939</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3373,7 +3367,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>BB_ET939_GL</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3382,7 +3376,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -3391,12 +3385,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3406,7 +3400,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3416,34 +3410,34 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>WILLY_CERES_NORD</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>ET939</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>BB_ET939_GL</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3452,7 +3446,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -3461,12 +3455,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-07-30 15:16:06</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-07-30 15:16:06</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3476,7 +3470,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3486,34 +3480,34 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3522,7 +3516,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -3531,12 +3525,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3546,7 +3540,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -3556,7 +3550,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -3568,22 +3562,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3592,7 +3586,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>14.5</v>
+        <v>1.7</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -3601,12 +3595,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-09-09 12:40:44</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-09-09 12:40:44</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3616,7 +3610,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3626,7 +3620,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
@@ -3638,22 +3632,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3662,7 +3656,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>1.7</v>
+        <v>14.5</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -3671,12 +3665,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-09 12:40:44</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-09 12:40:44</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3686,7 +3680,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3696,34 +3690,34 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TRANSUA</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AC566</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>BB_AC566_W</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3732,7 +3726,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3741,12 +3735,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-09-10 13:43:18</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-09-10 13:43:18</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3756,7 +3750,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3766,77 +3760,147 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-09-11 16:18:24</t>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>ABENGOUROU</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TRANSUA</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AC566</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>BB_AC566_W</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:55:54</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:55:54</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-13 16:18:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>ABIDJAN 02</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>JACQUEVIL</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>AC211</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>2G,4G</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>BB_AC211_GL</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G50" t="n">
+      <c r="G51" t="n">
         <v>1.5</v>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-09-11 10:19:32</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2026-09-11 10:19:32</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-09-13 08:49:17</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-13 08:49:17</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
         <is>
           <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="M51" t="inlineStr">
         <is>
           <t>ERICSSON</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>2026-09-11 16:18:24</t>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-09-13 16:18:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-14 00:20:42
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,14 +424,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TOUMODI_RAMBO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ET811</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,12 +538,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TOUMODI_RAMBO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ambient Temperature Unacceptable</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-13 08:02:57</t>
+          <t>2026-09-13 16:39:35</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-13 08:02:57</t>
+          <t>2026-09-13 16:39:35</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Specific Problem=Too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TOUMODI_RAMBO</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ET811</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TOUMODI_RAMBO</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-13 10:19:56</t>
+          <t>2026-09-13 19:53:08</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-13 10:19:56</t>
+          <t>2026-09-13 19:53:08</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=98/208, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=91/196, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>YOP_PORT-BOUET2_SIDOCO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>ET991</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>BB_ET991_GL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-13 10:55:19</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-13 10:55:19</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BAGOLIEOUA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC978</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BAGOLEHOUA</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-13 13:00:15</t>
+          <t>2026-09-13 09:03:50</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-13 13:00:15</t>
+          <t>2026-09-13 09:03:50</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-13 13:33:42</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-13 13:33:42</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,49 +836,49 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TOUMODI_RAMBO</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ET811</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TOUMODI_RAMBO</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-13 13:37:12</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-13 13:37:12</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,49 +903,49 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-13 14:21:56</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-13 14:21:56</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,49 +970,49 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-13 14:43:59</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-13 14:43:59</t>
+          <t>2026-09-12 10:49:55</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,49 +1037,49 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-13 15:19:39</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-13 15:19:39</t>
+          <t>2026-09-10 13:59:35</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,64 +1104,64 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YOP_PORT-BOUET2_SIDOCO</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ET991</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_ET991_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-13 21:59:45</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-13 21:59:45</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,17 +1171,17 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1193,27 +1193,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-13 09:03:50</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-13 09:03:50</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,24 +1449,24 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-12 10:49:55</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,24 +1516,24 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-10 13:59:35</t>
+          <t>2026-09-13 21:43:20</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,54 +1583,54 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ABOISSO_MUNICIPALITE</t>
+          <t>KOUN_ABRONZO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ET545</t>
+          <t>AC281</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Microwave</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ET545-ML6691</t>
+          <t>BB_AC281_W</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>High Temperature</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-13 14:34:55</t>
+          <t>2026-09-13 09:19:55</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-13 15:06:47</t>
+          <t>2026-09-13 11:52:44</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=MINILINK,MeContext=ET545-ML6691,ManagedElement=ET545-ML6691,NPU_1003=1/4 2578227022</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2578506393</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1650,54 +1650,57 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>TERMINAL_2</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ET903</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_ET903_WL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Indoor RAP Temperature Exceptional</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>245</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-13 15:52:28</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-13 15:52:28</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,64 +1710,67 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET903_WL,ManagedElement=BB_ET903_WL,Equipment=1,FieldReplaceableUnit=RD-1-3 2576221744</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>31</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1774,50 +1780,53 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>23</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1826,12 +1835,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 12:25:05</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 12:25:05</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1841,64 +1850,67 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>250</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1908,50 +1920,53 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>20</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1960,12 +1975,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-13 21:53:47</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-13 21:53:47</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1975,64 +1990,64 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=361, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2042,7 +2057,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2052,54 +2067,54 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2109,7 +2124,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2119,24 +2134,24 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>KOUN_ABRONZO</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AC281</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2146,27 +2161,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BB_AC281_W</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-13 09:19:55</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-13 11:52:44</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2176,7 +2191,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2578506393</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2186,43 +2201,40 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>245</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -2231,12 +2243,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2246,53 +2258,50 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>31</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -2301,12 +2310,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2316,67 +2325,64 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G29" t="n">
-        <v>23</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-09-13 21:47:20</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-09-13 23:36:39</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2386,53 +2392,50 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G30" t="n">
-        <v>250</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -2441,12 +2444,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-13 23:12:31</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-13 23:38:50</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2456,49 +2459,49 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2508,12 +2511,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-13 23:13:04</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-13 23:13:04</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2523,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2533,24 +2536,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>HERMANKONO_DIES</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC772</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2560,7 +2563,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>WAC772</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2575,12 +2578,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-13 23:17:06</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-13 23:17:06</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2590,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC772,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576053558</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2600,54 +2603,57 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>1.6</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2657,7 +2663,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2667,54 +2673,57 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1.8</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2724,7 +2733,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2734,54 +2743,57 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>WILLY_CERES_NORD</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET939</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_ET939_GL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1.7</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-07-30 15:16:06</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-07-30 15:16:06</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2791,7 +2803,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2801,54 +2813,57 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>2.1</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-13 15:28:11</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-13 15:28:11</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2858,7 +2873,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2868,54 +2883,57 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>1.7</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-13 15:38:16</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-13 15:38:16</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2925,7 +2943,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2935,54 +2953,57 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>14.5</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-13 15:41:38</t>
+          <t>2026-09-09 12:40:44</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-13 15:41:38</t>
+          <t>2026-09-09 12:40:44</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2992,7 +3013,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3002,54 +3023,57 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1.7</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-13 15:46:45</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-13 15:46:45</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3059,7 +3083,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3069,24 +3093,24 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3096,27 +3120,30 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1.9</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-13 15:52:02</t>
+          <t>2026-09-11 17:55:54</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-13 15:52:02</t>
+          <t>2026-09-11 17:55:54</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3126,7 +3153,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3136,771 +3163,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>YAMOUSSOUKRO</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>KOTIESSOU</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>AC763</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>RAN</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>AC763-OSmon</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Temperature is near limits</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>1970-01-04 21:21:22</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>1970-01-04 21:22:38</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2578639730</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>YAMOUSSOUKRO</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>KOTIESSOU</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>AC763</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>RAN</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>AC763-OSmon</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Temperature is near limits</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>1970-01-04 21:22:38</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>1970-01-04 21:22:38</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2578630038</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>GAGNOA</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>GOUDI</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>ET148</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>BB_ET148_GL</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-06-17 12:12:52</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2026-06-17 12:12:52</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-06-26 14:52:51</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-06-26 14:52:51</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>ABIDJAN 03</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>WILLY_CERES_NORD</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>ET939</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>BB_ET939_GL</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-07-30 15:16:06</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>2026-07-30 15:16:06</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ABIDJAN 01</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>ADAOU</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>AC548</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>BB_AC548_W</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>ET425</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>BB_ET425_GL</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>YOP_BAFOND</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>IM522</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>2G,3G</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>BB_IM522_GW</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-09-09 12:40:44</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>2026-09-09 12:40:44</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>TRANSUA</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>AC566</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>BB_AC566_W</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-09-11 17:55:54</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2026-09-11 17:55:54</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>JACQUEVIL</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>AC211</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>BB_AC211_GL</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-09-13 08:49:17</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2026-09-13 08:49:17</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>2026-09-13 16:18:25</t>
+          <t>2026-09-14 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-14 08:12:25
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-13 16:39:35</t>
+          <t>2026-09-14 00:22:15</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-13 16:39:35</t>
+          <t>2026-09-14 00:22:15</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-13 19:53:08</t>
+          <t>2026-09-14 06:34:09</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-13 19:53:08</t>
+          <t>2026-09-14 06:34:09</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=91/196, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YOP_PORT-BOUET2_SIDOCO</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ET991</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BB_ET991_GL</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-14 06:35:29</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-14 06:35:29</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-13 09:03:50</t>
+          <t>2026-09-14 07:51:46</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-13 09:03:50</t>
+          <t>2026-09-14 07:51:46</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-14 07:54:25</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-14 07:54:25</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,34 +836,34 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>YOP_PORT-BOUET2_SIDOCO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>ET991</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_ET991_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,39 +913,39 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-13 09:03:50</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-13 09:03:50</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-12 10:49:55</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,24 +1047,24 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-10 13:59:35</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,54 +1114,54 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-13 21:59:45</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-13 21:59:45</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,34 +1171,34 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-12 10:49:55</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 13:59:35</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,54 +1315,54 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-14 05:57:37</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-14 05:57:37</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,17 +1372,17 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
@@ -1461,12 +1461,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,24 +1516,24 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-13 21:43:20</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,34 +1583,34 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>KOUN_ABRONZO</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC281</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC281_W</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-13 09:19:55</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-13 11:52:44</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2578506393</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1650,57 +1650,54 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>245</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1710,67 +1707,64 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-13 21:43:20</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1780,53 +1774,50 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOUN_ABRONZO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC281</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC281_W</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>23</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1835,12 +1826,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-09-13 09:19:55</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-09-13 11:52:44</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1850,34 +1841,34 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2578506393</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1887,7 +1878,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1896,7 +1887,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1905,12 +1896,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1920,7 +1911,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1930,7 +1921,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
@@ -1942,12 +1933,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1957,7 +1948,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1966,21 +1957,21 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-13 21:53:47</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-13 21:53:47</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1990,7 +1981,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=361, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2000,54 +1991,57 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>23</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-10 12:25:05</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-10 12:25:05</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2057,50 +2051,53 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>250</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2109,12 +2106,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2124,64 +2121,67 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>20</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-13 21:53:47</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-13 21:53:47</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,34 +2191,34 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=361, RF Port=NULL</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2228,12 +2228,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2243,12 +2243,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,24 +2268,24 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>MASSADOUGOU_EST</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET816</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2295,27 +2295,27 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_ET816_W</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-09-14 07:36:39</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-14 07:36:39</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,MeContext=BB_ET816_W,ManagedElement=BB_ET816_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2578989727</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,24 +2335,24 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>MASSADOUGOU_EST</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>ET816</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2362,27 +2362,27 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>BB_ET816_W</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-13 21:47:20</t>
+          <t>2026-09-14 07:36:40</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-13 23:36:39</t>
+          <t>2026-09-14 07:36:40</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,MeContext=BB_ET816_W,ManagedElement=BB_ET816_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2578989726</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,54 +2402,54 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>MASSADOUGOU_EST</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>ET816</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>BB_ET816_GL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-13 23:12:31</t>
+          <t>2026-09-14 07:36:51</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-13 23:38:50</t>
+          <t>2026-09-14 07:36:51</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET816_GL,ManagedElement=BB_ET816_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2578993799</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,54 +2469,54 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>MASSADOUGOU_EST</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>ET816</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>BB_ET816_GL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-13 23:13:04</t>
+          <t>2026-09-14 07:36:52</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-13 23:13:04</t>
+          <t>2026-09-14 07:36:52</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET816_GL,ManagedElement=BB_ET816_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2578993798</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,54 +2536,54 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HERMANKONO_DIES</t>
+          <t>NASSIAN</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC772</t>
+          <t>AC546</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC772</t>
+          <t>BB_AC546_GL</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-13 23:17:06</t>
+          <t>2026-09-14 07:38:35</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-13 23:17:06</t>
+          <t>2026-09-14 07:38:35</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC772,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576053558</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC546_GL,ManagedElement=BB_AC546_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2578970857</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,24 +2603,24 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>NASSIAN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC546</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,30 +2630,27 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>BB_AC546_GL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>1.6</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-14 07:38:35</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-14 07:38:35</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2663,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC546_GL,ManagedElement=BB_AC546_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2579010198</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2673,57 +2670,54 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>1.8</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2733,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2743,57 +2737,54 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>WILLY_CERES_NORD</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET939</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET939_GL</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2803,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2813,24 +2804,24 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2840,30 +2831,27 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>2.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2873,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2883,7 +2871,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
@@ -2895,45 +2883,42 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2943,7 +2928,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2953,57 +2938,54 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>14.5</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-09 12:40:44</t>
+          <t>2026-09-14 06:03:17</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-09 12:40:44</t>
+          <t>2026-09-14 07:47:02</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3013,7 +2995,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3023,57 +3005,54 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-14 06:32:18</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-14 07:29:14</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3083,7 +3062,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3093,77 +3072,908 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-14 00:00:00</t>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DJOUROUTOU</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>AC787</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>WAC787</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-09-14 06:32:20</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:29:53</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>GBAPET</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AC781</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>WAC781</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-09-14 06:32:21</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:27:14</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MARC_AKWABA2</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ET001</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>RAN</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ET001-OSmon</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Temperature Outside Limits</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>1970-01-01 11:48:59</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>1970-01-01 11:48:59</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2578952089</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>GAGNOA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>GOUDI</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ET148</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BB_ET148_GL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>WILLY_CERES_NORD</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ET939</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BB_ET939_GL</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-07-30 15:16:06</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-07-30 15:16:06</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ADAOU</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>AC548</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BB_AC548_W</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>KOUWEIT_PIERRE_GADIE</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ET425</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>BB_ET425_GL</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-09-09 12:40:44</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-09-09 12:40:44</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>ABENGOUROU</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>TRANSUA</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>AC566</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>BB_AC566_W</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G40" t="n">
+      <c r="G50" t="n">
         <v>1.9</v>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>2026-09-11 17:55:54</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>2026-09-11 17:55:54</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="M50" t="inlineStr">
         <is>
           <t>ERICSSON</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>2026-09-14 00:00:00</t>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ABIDJAN 04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>YAKASSE_ME</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>AC543</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BB_AC543_GL</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-09-14 06:59:25</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-14 06:59:25</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC543_GL,ManagedElement=BB_AC543_GL,Equipment=1,FieldReplaceableUnit=RRUS-7_B1B3,RfPort=D 2579016354</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>DJIBI</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>AC061</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>BB_AC061_W</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:20:16</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:20:16</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,MeContext=BB_AC061_W,ManagedElement=BB_AC061_W,Equipment=1,FieldReplaceableUnit=RRU-6,RfPort=A 2578444735</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:00:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-15 12:05:30
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,14 +424,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-14 00:22:15</t>
+          <t>2026-09-14 14:30:55</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-14 00:22:15</t>
+          <t>2026-09-14 14:30:55</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC938</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-14 06:34:09</t>
+          <t>2026-09-14 19:57:44</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-14 06:34:09</t>
+          <t>2026-09-14 19:57:44</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=1, Board Type=UBBP, Current Board Temperature (C/F)=96/205, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,24 +645,24 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC938</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -682,17 +682,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-14 06:35:29</t>
+          <t>2026-09-14 19:59:24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-14 06:35:29</t>
+          <t>2026-09-14 19:59:24</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=103/217, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -712,24 +712,24 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC938</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-14 07:51:46</t>
+          <t>2026-09-14 19:59:38</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-14 07:51:46</t>
+          <t>2026-09-14 19:59:38</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=2, Board Type=UBBP, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -779,24 +779,24 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC938</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-14 07:54:25</t>
+          <t>2026-09-14 19:59:43</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-14 07:54:25</t>
+          <t>2026-09-14 19:59:43</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=3, Board Type=UBBP, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YOP_PORT-BOUET2_SIDOCO</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ET991</t>
+          <t>AC938</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_ET991_GL</t>
+          <t>KATIOLA_HOPITAL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-14 20:00:41</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-14 20:00:41</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,49 +903,49 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-13 09:03:50</t>
+          <t>2026-09-15 04:29:06</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-13 09:03:50</t>
+          <t>2026-09-15 04:29:06</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,49 +970,49 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-15 07:21:05</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-15 07:21:05</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,49 +1037,49 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-15 07:21:50</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-15 07:21:50</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,34 +1104,34 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>YOP_PORT-BOUET2_SIDOCO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET991</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET991_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,39 +1181,39 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-15 06:42:22</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-12 10:49:55</t>
+          <t>2026-09-15 06:42:22</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-10 13:59:35</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,54 +1315,54 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-14 05:57:37</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-14 05:57:37</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,34 +1372,34 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,24 +1449,24 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-12 10:49:55</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,24 +1516,24 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-10 13:59:35</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,54 +1583,54 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-15 07:04:14</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-15 07:04:14</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,64 +1640,64 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>KENEDY</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC382</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>WAC382</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>NTP Server Reachability Fault</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-15 07:51:23</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-15 07:51:23</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC06,SubNetwork=AORNC06_GROUP,MeContext=WAC382,ManagedElement=1,IpSystem=1,IpAccessHostEt=1,IpSyncRef=7 2579713179</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1717,54 +1717,54 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>KENEDY</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC382</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>WAC382</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>NTP Server Reachability Fault</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-15 07:51:23</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-13 21:43:20</t>
+          <t>2026-09-15 07:51:23</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC06,SubNetwork=AORNC06_GROUP,MeContext=WAC382,ManagedElement=1,IpSystem=1,IpAccessHostEt=1,IpSyncRef=8 2579710260</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1784,34 +1784,34 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KOUN_ABRONZO</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC281</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BB_AC281_W</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1826,12 +1826,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-13 09:19:55</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-13 11:52:44</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2578506393</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1851,57 +1851,54 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>245</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1911,67 +1908,64 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1981,53 +1975,50 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>23</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2036,12 +2027,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2051,67 +2042,64 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2121,53 +2109,50 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>20</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2176,12 +2161,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-13 21:53:47</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-13 21:53:47</t>
+          <t>2026-09-14 13:27:11</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,50 +2176,53 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=361, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>245</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -2243,12 +2231,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,64 +2246,67 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MASSADOUGOU_EST</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET816</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BB_ET816_W</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>31</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-14 07:36:39</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-14 07:36:39</t>
+          <t>2026-09-07 18:18:13</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,64 +2316,67 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,MeContext=BB_ET816_W,ManagedElement=BB_ET816_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2578989727</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MASSADOUGOU_EST</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET816</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BB_ET816_W</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>23</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-14 07:36:40</t>
+          <t>2026-09-10 12:25:05</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-14 07:36:40</t>
+          <t>2026-09-10 12:25:05</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,64 +2386,67 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,MeContext=BB_ET816_W,ManagedElement=BB_ET816_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2578989726</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MASSADOUGOU_EST</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ET816</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BB_ET816_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>250</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-14 07:36:51</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-14 07:36:51</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,64 +2456,67 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET816_GL,ManagedElement=BB_ET816_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2578993799</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MASSADOUGOU_EST</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ET816</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BB_ET816_GL</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>20</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-14 07:36:52</t>
+          <t>2026-09-15 07:49:48</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-14 07:36:52</t>
+          <t>2026-09-15 07:49:48</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,17 +2526,17 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET816_GL,ManagedElement=BB_ET816_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2578993798</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=351, RF Port=NULL</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
@@ -2548,42 +2548,42 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>NASSIAN</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC546</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BB_AC546_GL</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-14 07:38:35</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-14 07:38:35</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC546_GL,ManagedElement=BB_AC546_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2578970857</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,54 +2603,54 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NASSIAN</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC546</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BB_AC546_GL</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-14 07:38:35</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-14 07:38:35</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC546_GL,ManagedElement=BB_AC546_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2579010198</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
@@ -2749,12 +2749,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2779,12 +2779,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,24 +2804,24 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2846,12 +2846,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2871,24 +2871,24 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2913,12 +2913,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-09-15 06:14:38</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-15 07:58:13</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
@@ -2950,22 +2950,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-14 06:03:17</t>
+          <t>2026-09-15 06:45:32</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-14 07:47:02</t>
+          <t>2026-09-15 07:43:29</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
@@ -3017,22 +3017,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3047,12 +3047,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-14 06:32:18</t>
+          <t>2026-09-15 07:17:37</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-14 07:29:14</t>
+          <t>2026-09-15 07:17:37</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
@@ -3084,12 +3084,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3114,12 +3114,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-14 06:32:20</t>
+          <t>2026-09-15 07:39:59</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-14 07:29:53</t>
+          <t>2026-09-15 07:39:59</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3139,54 +3139,54 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>MARC_AKWABA2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>ET001</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>ET001-OSmon</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Temperature Outside Limits</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-14 06:32:21</t>
+          <t>1970-01-02 02:33:30</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-14 07:27:14</t>
+          <t>1970-01-02 02:33:30</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2579374016</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3206,54 +3206,57 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MARC_AKWABA2</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ET001</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ET001-OSmon</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Temperature Outside Limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1.6</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>1970-01-01 11:48:59</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>1970-01-01 11:48:59</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3263,7 +3266,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2578952089</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3273,24 +3276,24 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3300,7 +3303,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3309,7 +3312,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -3318,12 +3321,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3333,7 +3336,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3343,24 +3346,24 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>WILLY_CERES_NORD</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET939</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3370,7 +3373,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_ET939_GL</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3379,7 +3382,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -3388,12 +3391,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-07-30 15:16:06</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-07-30 15:16:06</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3403,7 +3406,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3413,34 +3416,34 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WILLY_CERES_NORD</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ET939</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BB_ET939_GL</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3449,7 +3452,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -3458,12 +3461,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3473,7 +3476,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3483,34 +3486,34 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3519,7 +3522,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -3528,12 +3531,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3543,7 +3546,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -3553,7 +3556,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
@@ -3565,22 +3568,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3589,7 +3592,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>1.7</v>
+        <v>14.5</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -3598,12 +3601,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-09 12:40:44</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-09 12:40:44</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3613,7 +3616,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3623,7 +3626,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
@@ -3635,22 +3638,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3659,7 +3662,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>14.5</v>
+        <v>1.7</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -3668,12 +3671,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-09-09 12:40:44</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-09-09 12:40:44</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3683,7 +3686,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3693,34 +3696,34 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3729,7 +3732,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3738,12 +3741,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-11 17:55:54</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-11 17:55:54</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3753,7 +3756,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3763,24 +3766,24 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TRANSUA</t>
+          <t>AGBAOU</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>AC566</t>
+          <t>ET119</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3790,7 +3793,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>BB_AC566_W</t>
+          <t>BB_ET119_W</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3799,7 +3802,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -3808,12 +3811,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-09-11 17:55:54</t>
+          <t>2026-09-15 03:43:57</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-09-11 17:55:54</t>
+          <t>2026-09-15 05:18:44</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3823,7 +3826,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET119_W,ManagedElement=BB_ET119_W,Equipment=1,FieldReplaceableUnit=RRUS-6,RfPort=A 2579646425</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -3833,34 +3836,34 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YAKASSE_ME</t>
+          <t>KOUN_ABRONZO</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>AC543</t>
+          <t>AC281</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>BB_AC543_GL</t>
+          <t>BB_AC281_W</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3869,7 +3872,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -3878,12 +3881,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-09-14 06:59:25</t>
+          <t>2026-09-15 04:14:45</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-09-14 06:59:25</t>
+          <t>2026-09-15 04:14:45</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3893,7 +3896,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC543_GL,ManagedElement=BB_AC543_GL,Equipment=1,FieldReplaceableUnit=RRUS-7_B1B3,RfPort=D 2579016354</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2579668347</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -3903,77 +3906,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-09-14 08:00:05</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>ABIDJAN 03</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>DJIBI</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>AC061</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>BB_AC061_W</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-09-14 07:20:16</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-09-14 07:20:16</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,MeContext=BB_AC061_W,ManagedElement=BB_AC061_W,Equipment=1,FieldReplaceableUnit=RRU-6,RfPort=A 2578444735</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>2026-09-14 08:00:05</t>
+          <t>2026-09-15 07:59:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-16 10:30:28
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,21 +424,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="208" customWidth="1" min="12" max="12"/>
+    <col width="204" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
@@ -518,32 +518,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>YOP_PORT-BOUET2_SIDOCO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>ET991</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>BB_ET991_GL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-15 11:44:11</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-15 11:44:11</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,49 +568,49 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-15 14:52:59</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-15 14:52:59</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,49 +635,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-15 15:46:41</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-15 15:46:41</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,34 +702,34 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YOP_PORT-BOUET2_SIDOCO</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ET991</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -739,12 +739,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_ET991_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -779,39 +779,39 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-15 06:42:22</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-15 06:42:22</t>
+          <t>2026-09-12 10:49:55</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DABOU_SODECI</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC932</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC932_W</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-15 15:30:31</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-15 15:30:31</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2577806954</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,54 +980,54 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-16 07:47:03</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-16 07:47:03</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,34 +1037,34 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-12 10:49:55</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,54 +1315,54 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ABOISSO_MUNICIPALITE</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ET545</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Microwave</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ET545-ML6691</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>High Temperature</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-15 15:45:42</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-15 15:45:42</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=MINILINK,MeContext=ET545-ML6691,ManagedElement=ET545-ML6691,NPU_1003=1/4 2578227022</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,54 +1382,54 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2PLTX_KAVOKIVA</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC998</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>WAC998</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>NTP Server Reachability Fault</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-15 13:13:54</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-15 15:56:18</t>
+          <t>2026-09-14 13:27:11</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC01,SubNetwork=ABRNC01_GROUP,MeContext=WAC998,ManagedElement=1,IpSystem=1,IpAccessHostEt=1,IpSyncRef=8 2576218395</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,40 +1449,43 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2PLTX_KAVOKIVA</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC998</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>WAC998</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>NTP Server Reachability Fault</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>250</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1491,12 +1494,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-15 15:56:18</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-15 15:56:18</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,64 +1509,67 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC01,SubNetwork=ABRNC01_GROUP,MeContext=WAC998,ManagedElement=1,IpSystem=1,IpAccessHostEt=1,IpSyncRef=7 2576224184</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>31</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,64 +1579,67 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>245</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,64 +1649,67 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>31</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,50 +1719,53 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>20</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1759,12 +1774,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-16 07:07:49</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-16 07:07:49</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1774,50 +1789,53 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=431, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>ADJAHUI_GATL</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>ET974</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>ADJAHUI_GATL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>20</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1826,12 +1844,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-16 07:58:03</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-16 07:58:03</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1841,64 +1859,64 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=405, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-14 13:27:11</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1908,7 +1926,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1918,57 +1936,54 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOUM_INCHALLAH</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET393</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_ET393_GL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>245</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-16 06:30:51</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-16 06:30:51</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1978,67 +1993,64 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET393_GL,ManagedElement=BB_ET393_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580112078</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOUM_INCHALLAH</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET393</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_ET393_GL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>31</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-16 06:30:51</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-07 18:18:13</t>
+          <t>2026-09-16 06:30:51</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2048,67 +2060,64 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET393_GL,ManagedElement=BB_ET393_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580112077</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>23</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-10 12:25:05</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2118,53 +2127,50 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=23, Output Power (0.1 dBm)=372, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>250</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2173,12 +2179,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2188,67 +2194,64 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>20</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-15 14:39:49</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-15 14:39:49</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,34 +2261,34 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2295,12 +2298,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2310,12 +2313,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2328,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,54 +2338,54 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CIMAF</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET090</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BB_ET090_GL</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-15 15:48:34</t>
+          <t>2026-09-16 05:54:10</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-15 15:48:34</t>
+          <t>2026-09-16 07:48:04</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2395,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET090_GL,ManagedElement=BB_ET090_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2579843589</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,54 +2405,54 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CIMAF</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ET090</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BB_ET090_GL</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-15 15:48:34</t>
+          <t>2026-09-16 06:56:45</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-15 15:48:34</t>
+          <t>2026-09-16 07:53:45</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2462,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET090_GL,ManagedElement=BB_ET090_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2579832865</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,54 +2472,54 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CIMAF</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ET090</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BB_ET090_W</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-15 15:48:35</t>
+          <t>2026-09-16 07:30:39</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-15 15:48:35</t>
+          <t>2026-09-16 07:30:39</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2529,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET090_W,ManagedElement=BB_ET090_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2579832864</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,24 +2539,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CIMAF</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ET090</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,27 +2566,27 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BB_ET090_W</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-15 15:48:35</t>
+          <t>2026-09-16 07:47:11</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-15 15:48:35</t>
+          <t>2026-09-16 07:47:11</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2596,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET090_W,ManagedElement=BB_ET090_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2579843586</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,54 +2606,57 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>1.6</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2666,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,54 +2676,57 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1.8</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2736,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,54 +2746,57 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>WILLY_CERES_NORD</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>ET939</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BB_ET939_GL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1.7</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-07-30 15:16:06</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-07-30 15:16:06</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2806,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,24 +2816,24 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2831,27 +2843,30 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>2.1</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2861,7 +2876,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2871,7 +2886,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
@@ -2883,42 +2898,45 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>1.7</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-15 12:57:49</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-15 15:43:00</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2928,7 +2946,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2938,54 +2956,57 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MARC_AKWABA2</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET001</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ET001-OSmon</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Temperature Outside Limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1.7</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1970-01-02 21:41:42</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>1970-01-02 21:42:11</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2995,7 +3016,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2579935518</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3005,54 +3026,57 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KOTIESSOU</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AC763</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>AC763-OSmon</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1.9</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>1970-01-06 21:28:47</t>
+          <t>2026-09-11 17:55:54</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>1970-01-06 21:29:08</t>
+          <t>2026-09-11 17:55:54</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3062,7 +3086,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2579932583</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3072,54 +3096,57 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KOTIESSOU</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC763</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>AC763-OSmon</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>11.6</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>1970-01-06 21:29:08</t>
+          <t>2026-09-15 12:26:40</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>1970-01-06 21:29:08</t>
+          <t>2026-09-15 12:26:40</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3129,7 +3156,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2579914022</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3139,40 +3166,43 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>GESTOCI</t>
+          <t>KOUN_ABRONZO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC094</t>
+          <t>AC281</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>IP</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>AC094PER6273_01</t>
+          <t>BB_AC281_W</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Transceiver Temperature High Warning</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>6</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -3181,12 +3211,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-15 09:11:08</t>
+          <t>2026-09-16 05:13:51</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-15 09:54:41</t>
+          <t>2026-09-16 05:13:51</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3196,7 +3226,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=ROUTER,MeContext=AC094PER6273_01,ManagedElement=1,interfaces=1,interface=2/1 2576388604</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2579668347</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3206,847 +3236,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>GAGNOA</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>GOUDI</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>ET148</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>BB_ET148_GL</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-06-17 12:12:52</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2026-06-17 12:12:52</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-06-26 14:52:51</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2026-06-26 14:52:51</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ABIDJAN 03</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>WILLY_CERES_NORD</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>ET939</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>BB_ET939_GL</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-07-30 15:16:06</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-07-30 15:16:06</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>ABIDJAN 01</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>ADAOU</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>AC548</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>BB_AC548_W</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>ET425</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>BB_ET425_GL</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>TRANSUA</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>AC566</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>BB_AC566_W</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-09-11 17:55:54</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>2026-09-11 17:55:54</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>GAGNOA</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>AGBAOU</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>ET119</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>BB_ET119_W</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-09-15 10:17:53</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>2026-09-15 10:17:53</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET119_W,ManagedElement=BB_ET119_W,Equipment=1,FieldReplaceableUnit=RRUS-6,RfPort=A 2579646425</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>YOP_BAFOND</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>IM522</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>2G,3G</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>BB_IM522_GW</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-09-15 12:26:40</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2026-09-15 12:26:40</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>ABIDJAN 03</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>STAR_2</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>AC365</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>BB_AC365_GL</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-09-15 13:25:31</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2026-09-15 13:25:31</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC365_GL,ManagedElement=BB_AC365_GL,Equipment=1,FieldReplaceableUnit=RRUS-9_B3,RfPort=B 2579844001</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>SONGON_BEL_HORIZON</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>ET815</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>BB_ET815_GL</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-09-15 14:10:55</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-09-15 14:10:55</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2578625791</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>JACQUEVIL</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>AC211</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>BB_AC211_GL</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-09-15 14:41:13</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2026-09-15 14:41:13</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>2026-09-15 16:00:37</t>
+          <t>2026-09-16 07:59:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-16 16:29:40
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,14 +424,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
@@ -518,32 +518,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YOP_PORT-BOUET2_SIDOCO</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ET991</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BB_ET991_GL</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-16 12:15:46</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-12 20:26:53</t>
+          <t>2026-09-16 12:15:46</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,49 +568,49 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-16 12:40:02</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-16 12:40:02</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,49 +635,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-16 15:43:13</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-16 15:43:13</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-16 15:47:14</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-16 15:47:14</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,34 +769,34 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>YOP_PORT-BOUET2_SIDOCO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET991</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -806,12 +806,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET991_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-12 10:49:55</t>
+          <t>2026-09-12 20:26:53</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET991_GL,ManagedElement=BB_ET991_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B1B3B7 2576086477</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-16 08:34:04</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-16 08:34:04</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,39 +913,39 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>DABOU_SODECI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC932</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC932_W</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-16 12:44:19</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-16 12:44:19</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2577806954</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,54 +980,54 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-16 07:47:03</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-16 07:47:03</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,34 +1037,34 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,39 +1315,39 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>TERMINAL_2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>ET903</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_ET903_WL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Indoor RAP Temperature Exceptional</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-16 15:43:35</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-16 15:43:35</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET903_WL,ManagedElement=BB_ET903_WL,Equipment=1,FieldReplaceableUnit=RD-1-3 2576221744</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,54 +1382,54 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>GUIGUEDOU</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC776</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>WAC776</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>NTP Server Reachability Fault</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-16 14:58:17</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-14 13:27:11</t>
+          <t>2026-09-16 15:55:20</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WAC776,ManagedElement=1,IpSystem=1,IpAccessHostEt=1,IpSyncRef=7 2576049659</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
@@ -1461,31 +1461,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>GUIGUEDOU</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC776</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>WAC776</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>250</v>
+          <t>NTP Server Reachability Fault</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1494,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-16 15:55:20</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-16 15:55:20</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1509,67 +1506,64 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WAC776,ManagedElement=1,IpSystem=1,IpAccessHostEt=1,IpSyncRef=8 2576053654</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-16 05:28:25</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-16 05:28:25</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1579,67 +1573,64 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>245</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-16 05:28:25</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-16 05:28:25</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1649,67 +1640,64 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-16 05:28:25</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-16 05:28:25</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1719,53 +1707,50 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>20</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1774,12 +1759,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-16 07:07:49</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-16 07:07:49</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1789,53 +1774,50 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=431, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ADJAHUI_GATL</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ET974</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ADJAHUI_GATL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>20</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1844,12 +1826,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-16 07:58:03</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-16 07:58:03</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1859,64 +1841,64 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=405, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-14 13:27:11</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1926,7 +1908,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1936,54 +1918,57 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KOUM_INCHALLAH</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET393</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BB_ET393_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>250</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-16 06:30:51</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-16 06:30:51</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1993,64 +1978,67 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET393_GL,ManagedElement=BB_ET393_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580112078</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KOUM_INCHALLAH</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET393</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BB_ET393_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>31</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-16 06:30:51</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-16 06:30:51</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2060,50 +2048,53 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET393_GL,ManagedElement=BB_ET393_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580112077</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>245</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2112,12 +2103,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2127,50 +2118,53 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>31</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2179,12 +2173,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-16 05:28:25</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2194,64 +2188,67 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>20</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-16 14:27:49</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-16 14:27:49</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2261,34 +2258,34 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=351, RF Port=NULL</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2298,12 +2295,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2313,12 +2310,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2328,7 +2325,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2338,7 +2335,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
@@ -2350,12 +2347,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2365,7 +2362,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2380,12 +2377,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-16 05:54:10</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-16 07:48:04</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2395,7 +2392,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2405,7 +2402,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
@@ -2417,12 +2414,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2432,7 +2429,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2447,12 +2444,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-16 06:56:45</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-16 07:53:45</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2462,7 +2459,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2472,7 +2469,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
@@ -2484,22 +2481,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2514,12 +2511,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-16 07:30:39</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-16 07:30:39</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2529,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2539,24 +2536,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2566,7 +2563,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2581,12 +2578,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-16 07:47:11</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-16 07:47:11</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2596,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2606,57 +2603,54 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>1.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-16 14:54:28</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-16 15:50:22</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2666,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2676,57 +2670,54 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>1.8</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-09-16 15:13:33</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-09-16 15:13:33</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2736,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2746,57 +2737,54 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>WILLY_CERES_NORD</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET939</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET939_GL</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-09-16 15:33:07</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-09-16 15:33:07</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2806,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2816,57 +2804,54 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>2.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-16 15:57:20</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-16 15:57:20</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2876,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2886,57 +2871,54 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-16 15:57:43</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-16 15:57:43</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2946,7 +2928,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2956,57 +2938,54 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>ANGRE_CIT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET084</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>ET084-OSmon</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>1.7</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2007-01-31 15:04:46</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2007-01-31 15:04:46</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3016,7 +2995,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=TCU,MeContext=ET084-OSmon,STN=0,Equipment=0 2580476186</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3026,57 +3005,54 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TRANSUA</t>
+          <t>KOTIESSOU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AC566</t>
+          <t>AC763</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_AC566_W</t>
+          <t>AC763-OSmon</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>1.9</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-11 17:55:54</t>
+          <t>1970-01-07 18:01:49</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-11 17:55:54</t>
+          <t>1970-01-07 20:56:14</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3086,7 +3062,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2580414247</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3096,57 +3072,54 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>KOTIESSOU</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>AC763</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>AC763-OSmon</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>11.6</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-15 12:26:40</t>
+          <t>1970-01-07 20:56:14</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-15 12:26:40</t>
+          <t>1970-01-07 20:56:14</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3156,7 +3129,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2580450025</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3166,77 +3139,704 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-16 07:59:54</t>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>GESTOCI</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AC094</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>AC094PER6273_01</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Transceiver Temperature High Warning</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-09-16 10:25:52</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-09-16 10:54:27</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SubNetwork=ROUTER,MeContext=AC094PER6273_01,ManagedElement=1,interfaces=1,interface=2/1 2576388604</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>GAGNOA</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>GOUDI</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ET148</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BB_ET148_GL</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>WILLY_CERES_NORD</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ET939</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BB_ET939_GL</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-07-30 15:16:06</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-07-30 15:16:06</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ADAOU</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AC548</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BB_AC548_W</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>KOUWEIT_PIERRE_GADIE</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ET425</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BB_ET425_GL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>ABENGOUROU</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>KOUN_ABRONZO</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>AC281</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TRANSUA</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AC566</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>BB_AC281_W</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BB_AC566_W</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G41" t="n">
-        <v>6</v>
-      </c>
-      <c r="H41" t="inlineStr">
+      <c r="G48" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2026-09-16 05:13:51</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>2026-09-16 05:13:51</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC281_W,ManagedElement=BB_AC281_W,Equipment=1,FieldReplaceableUnit=RRUS-4,RfPort=A 2579668347</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>2026-09-16 07:59:54</t>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:55:54</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:55:54</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-09-15 12:26:40</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-09-15 12:26:40</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>JACQUEVIL</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AC211</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>BB_AC211_GL</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-09-16 09:25:37</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-09-16 09:25:37</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:18:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-17 16:33:21
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,15 +424,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
@@ -518,27 +518,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-17 06:15:24</t>
+          <t>2026-09-17 11:15:21</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-17 06:15:24</t>
+          <t>2026-09-17 11:15:21</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,39 +578,39 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-17 12:00:48</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-17 12:00:48</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,49 +635,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-17 14:03:44</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-17 14:03:44</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-17 14:47:24</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-17 14:47:24</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>GOBAZRA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET502</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>GOBAZRA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-17 15:24:37</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-16 18:17:14</t>
+          <t>2026-09-17 15:24:37</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,49 +836,49 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-17 08:00:47</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-17 08:00:47</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,39 +913,39 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>DABOU_SODECI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC932</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC932_W</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-17 09:35:25</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-17 09:35:25</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2577806954</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,54 +980,54 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-17 07:29:27</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-17 07:29:27</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,34 +1037,34 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-16 18:17:14</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,54 +1382,54 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>KORHOGO</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>BOLONA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>ET922</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BOLONA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-17 14:40:50</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-17 01:12:29</t>
+          <t>2026-09-17 14:40:50</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,67 +1439,64 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1509,67 +1506,64 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>245</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1579,67 +1573,64 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1649,67 +1640,64 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1719,53 +1707,50 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>20</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1774,12 +1759,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-17 06:49:50</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-17 06:49:50</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1789,64 +1774,64 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=353, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-17 01:12:29</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1856,7 +1841,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1866,54 +1851,57 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC155</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BB_AC155_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>250</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-16 20:58:05</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-16 20:58:05</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1923,64 +1911,67 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC155_GL,ManagedElement=BB_AC155_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 -2</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KOTCHERI</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET151</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BB_ET151_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>245</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-16 20:58:05</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-16 20:58:05</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1990,64 +1981,67 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET151_GL,ManagedElement=BB_ET151_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 -2</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>31</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:00</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:00</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2057,64 +2051,67 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>31</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:06</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:06</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2124,64 +2121,67 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>20</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:32</t>
+          <t>2026-09-17 13:37:50</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:32</t>
+          <t>2026-09-17 13:37:50</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,34 +2191,34 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=359, RF Port=NULL</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2228,27 +2228,27 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-17 06:04:56</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-17 06:04:56</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
@@ -2280,42 +2280,42 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>LAC</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC155</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>BB_AC155_GL</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-16 20:58:05</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-16 20:58:05</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC155_GL,ManagedElement=BB_AC155_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 -2</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,54 +2335,54 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>KOTCHERI</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET151</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>BB_ET151_GL</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-16 20:58:05</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-16 20:58:05</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET151_GL,ManagedElement=BB_ET151_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 -2</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
@@ -2414,42 +2414,42 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-17 06:01:00</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-17 06:01:00</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,54 +2469,54 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-09-17 06:01:06</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-17 06:01:06</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
@@ -2548,12 +2548,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,27 +2563,27 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-17 05:52:51</t>
+          <t>2026-09-17 06:01:32</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-17 07:36:33</t>
+          <t>2026-09-17 06:01:32</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
@@ -2615,42 +2615,42 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-17 06:37:07</t>
+          <t>2026-09-17 06:04:56</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-17 07:35:21</t>
+          <t>2026-09-17 06:04:56</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,54 +2670,54 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>KOUM_INCHALLAH</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>ET393</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>BB_ET393_GL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-17 06:37:12</t>
+          <t>2026-09-17 14:52:54</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-17 07:34:44</t>
+          <t>2026-09-17 14:52:54</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET393_GL,ManagedElement=BB_ET393_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580112078</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,24 +2737,24 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>KOUM_INCHALLAH</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>ET393</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2764,30 +2764,27 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>BB_ET393_GL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1.6</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-17 14:52:54</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-17 14:52:54</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2797,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET393_GL,ManagedElement=BB_ET393_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580112077</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2807,57 +2804,54 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>1.8</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2867,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2877,57 +2871,54 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>WILLY_CERES_NORD</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ET939</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_ET939_GL</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-07-30 15:16:06</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2937,7 +2928,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET939_GL,ManagedElement=BB_ET939_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=E 2568853076</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2947,24 +2938,24 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2974,30 +2965,27 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>2.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3007,7 +2995,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3017,7 +3005,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
@@ -3029,45 +3017,42 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3077,7 +3062,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3087,57 +3072,54 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>KM4</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC098</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>LAC098</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-17 15:19:17</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-17 15:19:17</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3147,7 +3129,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC098,ManagedElement=1,TransportNetwork=1,Synchronization=1 2579063722</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3157,24 +3139,24 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TRANSUA</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC566</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3184,30 +3166,27 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BB_AC566_W</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>1.9</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-11 17:55:54</t>
+          <t>2026-09-17 15:31:56</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-11 17:55:54</t>
+          <t>2026-09-17 15:31:56</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3217,7 +3196,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3227,57 +3206,54 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>11.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-15 12:26:40</t>
+          <t>2026-09-17 15:32:16</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-15 12:26:40</t>
+          <t>2026-09-17 15:32:16</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3287,7 +3263,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3297,77 +3273,972 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:07</t>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BOUBOURY</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AC534</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>WAC534</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:37:19</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:37:19</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>GBAPET</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AC781</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>WAC781</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:54:41</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:54:41</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>GBAPET</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AC781</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LAC781</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:57:41</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:57:41</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>GESTOCI</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>AC094</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>AC094PER6273_01</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Transceiver Temperature High Warning</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-09-17 08:35:52</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:54:40</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SubNetwork=ROUTER,MeContext=AC094PER6273_01,ManagedElement=1,interfaces=1,interface=2/1 2576388604</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>DALOA</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>DAL_BSC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>AC904</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>CONTROLER-2G/3G</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>DAMBSC13</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Transmission Resource Pool Ping Packet Loss</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:40:02</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:40:02</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Subrack No.=0, Slot No.=4, IP Address in the Transmission Resource Pool=10.188.17.57</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>HUAWEI</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>GAGNOA</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>GOUDI</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ET148</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BB_ET148_GL</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ADAOU</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AC548</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>BB_AC548_W</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>KOUWEIT_PIERRE_GADIE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ET425</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BB_ET425_GL</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-09-15 12:26:40</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-09-15 12:26:40</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>JACQUEVIL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>AC211</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>BB_AC211_GL</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-09-17 09:27:16</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-09-17 09:27:16</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>ABIDJAN 03</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>STAR_2</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>AC365</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>2G,4G</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>BB_AC365_GL</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G43" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="H43" t="inlineStr">
+      <c r="G55" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H55" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-09-16 16:34:59</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2026-09-16 16:34:59</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:16:28</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:16:28</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC365_GL,ManagedElement=BB_AC365_GL,Equipment=1,FieldReplaceableUnit=RRUS-9_B3,RfPort=B 2579844001</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M55" t="inlineStr">
         <is>
           <t>ERICSSON</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-09-17 08:00:07</t>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ABENGOUROU</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>TRANSUA</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>AC566</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>BB_AC566_W</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:34:49</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:34:49</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:15:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-18 00:30:20
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,15 +424,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
@@ -518,27 +518,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-17 11:15:21</t>
+          <t>2026-09-17 14:03:44</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-17 11:15:21</t>
+          <t>2026-09-17 14:03:44</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-17 12:00:48</t>
+          <t>2026-09-17 18:57:38</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-17 12:00:48</t>
+          <t>2026-09-17 18:57:38</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-17 14:03:44</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-17 14:03:44</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-17 14:47:24</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-17 14:47:24</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GOBAZRA</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET502</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>GOBAZRA</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-17 15:24:37</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-17 15:24:37</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,49 +836,49 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:47</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-17 08:00:47</t>
+          <t>2026-09-16 18:17:14</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,39 +913,39 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DABOU_SODECI</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC932</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC932_W</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-17 09:35:25</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-17 09:35:25</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2577806954</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,24 +1047,24 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-16 18:17:14</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,54 +1382,54 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KORHOGO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BOLONA</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ET922</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BOLONA</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-17 14:40:50</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-17 14:40:50</t>
+          <t>2026-09-17 22:09:40</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,64 +1439,67 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>250</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,64 +1509,67 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>245</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,64 +1579,67 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>31</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,64 +1649,67 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>31</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,50 +1719,53 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>20</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1759,12 +1774,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-17 22:07:50</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-17 22:07:50</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1774,64 +1789,64 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=355, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-17 01:12:29</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1841,7 +1856,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1851,57 +1866,54 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>250</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-17 06:01:00</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-17 06:01:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1911,67 +1923,64 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>245</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-17 06:01:06</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-17 06:01:06</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1981,67 +1990,64 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>31</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-17 06:01:32</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-17 06:01:32</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2051,67 +2057,64 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>31</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-17 06:04:56</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-17 06:04:56</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2121,67 +2124,64 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>DAKOURITROHOUIN</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET093</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BB_ET093_GL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>20</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-17 13:37:50</t>
+          <t>2026-09-17 23:13:15</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-17 13:37:50</t>
+          <t>2026-09-17 23:50:27</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,34 +2191,34 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=359, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET093_GL,ManagedElement=BB_ET093_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580013881</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>DAKOURITROHOUIN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET093</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2228,27 +2228,27 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>BB_ET093_W</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-17 23:13:16</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-17 23:50:29</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET093_W,ManagedElement=BB_ET093_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580032860</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,34 +2268,34 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>LAC</t>
+          <t>DAKOURITROHOUIN</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC155</t>
+          <t>ET093</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BB_AC155_GL</t>
+          <t>BB_ET093_W</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2310,12 +2310,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-16 20:58:05</t>
+          <t>2026-09-17 23:13:16</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-16 20:58:05</t>
+          <t>2026-09-17 23:50:29</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC155_GL,ManagedElement=BB_AC155_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 -2</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET093_W,ManagedElement=BB_ET093_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580032861</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
@@ -2347,12 +2347,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>KOTCHERI</t>
+          <t>DAKOURITROHOUIN</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET151</t>
+          <t>ET093</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BB_ET151_GL</t>
+          <t>BB_ET093_GL</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2377,12 +2377,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-16 20:58:05</t>
+          <t>2026-09-17 23:13:16</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-16 20:58:05</t>
+          <t>2026-09-17 23:50:28</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET151_GL,ManagedElement=BB_ET151_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 -2</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET093_GL,ManagedElement=BB_ET093_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580013882</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,24 +2402,24 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>GUIGUEDOU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC776</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>BB_AC776_GL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:00</t>
+          <t>2026-09-17 23:13:17</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:00</t>
+          <t>2026-09-17 23:50:28</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC776_GL,ManagedElement=BB_AC776_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580037504</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,24 +2469,24 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>GUIGUEDOU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC776</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>BB_AC776_GL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2511,12 +2511,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:06</t>
+          <t>2026-09-17 23:13:17</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:06</t>
+          <t>2026-09-17 23:50:28</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC776_GL,ManagedElement=BB_AC776_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580037505</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
@@ -2548,12 +2548,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,27 +2563,27 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:32</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:32</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
@@ -2615,12 +2615,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,27 +2630,27 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-17 06:04:56</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-17 06:04:56</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,54 +2670,54 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>KOUM_INCHALLAH</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ET393</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BB_ET393_GL</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-17 14:52:54</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-17 14:52:54</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET393_GL,ManagedElement=BB_ET393_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580112078</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,54 +2737,54 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KOUM_INCHALLAH</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET393</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET393_GL</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-17 14:52:54</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-17 14:52:54</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET393_GL,ManagedElement=BB_ET393_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580112077</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,54 +2804,57 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>1.6</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2861,7 +2864,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2871,54 +2874,57 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>1.8</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2928,7 +2934,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2938,24 +2944,24 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2965,27 +2971,30 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>2.1</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2995,7 +3004,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3005,7 +3014,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
@@ -3017,42 +3026,45 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1.7</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3062,7 +3074,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3072,54 +3084,57 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KM4</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC098</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>LAC098</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1.7</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-17 15:19:17</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-17 15:19:17</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3129,7 +3144,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC098,ManagedElement=1,TransportNetwork=1,Synchronization=1 2579063722</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3139,54 +3154,57 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>11.6</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-17 15:31:56</t>
+          <t>2026-09-15 12:26:40</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-17 15:31:56</t>
+          <t>2026-09-15 12:26:40</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3196,7 +3214,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3206,1039 +3224,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>PARA</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>ET178</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>WET178</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:32:16</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:32:16</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>BOUBOURY</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>AC534</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>WAC534</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:37:19</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:37:19</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>GBAPET</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>AC781</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>WAC781</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:54:41</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:54:41</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>GBAPET</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>AC781</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>4G</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>LAC781</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:57:41</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:57:41</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ABIDJAN 01</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>GESTOCI</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>AC094</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>IP</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>AC094PER6273_01</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Transceiver Temperature High Warning</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-09-17 08:35:52</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2026-09-17 10:54:40</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>SubNetwork=ROUTER,MeContext=AC094PER6273_01,ManagedElement=1,interfaces=1,interface=2/1 2576388604</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>DALOA</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>DAL_BSC</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>AC904</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>CONTROLER-2G/3G</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>DAMBSC13</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Transmission Resource Pool Ping Packet Loss</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:40:02</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:40:02</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>Subrack No.=0, Slot No.=4, IP Address in the Transmission Resource Pool=10.188.17.57</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>HUAWEI</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>GAGNOA</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>GOUDI</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>ET148</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>BB_ET148_GL</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-06-17 12:12:52</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>2026-06-17 12:12:52</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-06-26 14:52:51</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>2026-06-26 14:52:51</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>ABIDJAN 01</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>ADAOU</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>AC548</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>BB_AC548_W</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>ET425</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>BB_ET425_GL</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>YOP_BAFOND</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>IM522</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>2G,3G</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>BB_IM522_GW</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-09-15 12:26:40</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2026-09-15 12:26:40</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>JACQUEVIL</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>AC211</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>BB_AC211_GL</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>2026-09-17 09:27:16</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>2026-09-17 09:27:16</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ABIDJAN 03</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>STAR_2</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>AC365</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>BB_AC365_GL</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>2026-09-17 13:16:28</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>2026-09-17 13:16:28</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC365_GL,ManagedElement=BB_AC365_GL,Equipment=1,FieldReplaceableUnit=RRUS-9_B3,RfPort=B 2579844001</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>TRANSUA</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>AC566</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>BB_AC566_W</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>2026-09-17 14:34:49</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>2026-09-17 14:34:49</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>2026-09-17 16:15:03</t>
+          <t>2026-09-18 00:15:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-18 08:20:46
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,10 +424,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-17 14:03:44</t>
+          <t>2026-09-18 06:24:01</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-17 14:03:44</t>
+          <t>2026-09-18 06:24:01</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-17 18:57:38</t>
+          <t>2026-09-18 07:13:07</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-17 18:57:38</t>
+          <t>2026-09-18 07:13:07</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-16 18:17:14</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -1047,54 +1047,54 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-18 06:57:02</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-18 06:57:02</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,17 +1104,17 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -1126,12 +1126,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-17 22:09:40</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,57 +1449,54 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-17 22:09:40</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1509,34 +1506,34 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1546,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1555,7 +1552,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1564,12 +1561,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1579,7 +1576,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1589,7 +1586,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1622,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>31</v>
+        <v>245</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1649,7 +1646,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1659,7 +1656,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1716,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1729,7 +1726,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -1741,12 +1738,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1756,7 +1753,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1765,21 +1762,21 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-17 22:07:50</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-17 22:07:50</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1789,7 +1786,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=355, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1799,54 +1796,57 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>20</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-18 07:57:51</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-18 07:57:51</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1856,64 +1856,64 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=356, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:00</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:00</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -1975,12 +1975,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:06</t>
+          <t>2026-09-18 06:14:08</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:06</t>
+          <t>2026-09-18 06:14:08</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -2042,12 +2042,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:32</t>
+          <t>2026-09-18 06:15:23</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-17 06:01:32</t>
+          <t>2026-09-18 06:15:23</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -2089,12 +2089,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2109,12 +2109,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-17 06:04:56</t>
+          <t>2026-09-18 06:16:43</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-17 06:04:56</t>
+          <t>2026-09-18 06:16:43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2134,34 +2134,34 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DAKOURITROHOUIN</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET093</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BB_ET093_GL</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2176,12 +2176,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-17 23:13:15</t>
+          <t>2026-09-18 06:22:29</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-17 23:50:27</t>
+          <t>2026-09-18 06:22:29</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET093_GL,ManagedElement=BB_ET093_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580013881</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2201,24 +2201,24 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DAKOURITROHOUIN</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET093</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2228,27 +2228,27 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BB_ET093_W</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-17 23:13:16</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-17 23:50:29</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET093_W,ManagedElement=BB_ET093_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580032860</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,24 +2268,24 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DAKOURITROHOUIN</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET093</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2295,27 +2295,27 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BB_ET093_W</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-17 23:13:16</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-17 23:50:29</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET093_W,ManagedElement=BB_ET093_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580032861</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,54 +2335,54 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DAKOURITROHOUIN</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET093</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BB_ET093_GL</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-17 23:13:16</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-17 23:50:28</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET093_GL,ManagedElement=BB_ET093_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580013882</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,54 +2402,54 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GUIGUEDOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC776</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BB_AC776_GL</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-17 23:13:17</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-17 23:50:28</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC776_GL,ManagedElement=BB_AC776_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580037504</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,54 +2469,54 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GUIGUEDOU</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC776</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BB_AC776_GL</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-17 23:13:17</t>
+          <t>2026-09-18 05:28:49</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-17 23:50:28</t>
+          <t>2026-09-18 07:15:14</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC776_GL,ManagedElement=BB_AC776_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580037505</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -2548,12 +2548,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2578,12 +2578,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-18 06:36:18</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-18 07:29:42</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -2615,12 +2615,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-18 06:43:00</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-18 07:37:45</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -2682,22 +2682,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-18 06:47:49</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-18 07:45:04</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,54 +2737,57 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1.6</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2797,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,24 +2807,24 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2831,7 +2834,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2840,7 +2843,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2849,12 +2852,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2864,7 +2867,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2874,34 +2877,34 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2910,7 +2913,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2919,12 +2922,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2934,7 +2937,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2944,34 +2947,34 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2980,7 +2983,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2989,12 +2992,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3004,7 +3007,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3014,7 +3017,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -3026,12 +3029,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3041,7 +3044,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3059,12 +3062,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3074,7 +3077,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3084,7 +3087,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
@@ -3096,22 +3099,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3120,7 +3123,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1.7</v>
+        <v>11.6</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -3129,12 +3132,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-15 12:26:40</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-15 12:26:40</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3144,7 +3147,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3154,34 +3157,34 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3190,7 +3193,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>11.6</v>
+        <v>1.9</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -3199,12 +3202,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-15 12:26:40</t>
+          <t>2026-09-18 00:08:08</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-15 12:26:40</t>
+          <t>2026-09-18 00:08:08</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3214,7 +3217,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3224,7 +3227,77 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-18 00:15:16</t>
+          <t>2026-09-18 08:00:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>DJIBI</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>AC061</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BB_AC061_W</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-09-18 06:37:09</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-09-18 06:37:09</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,MeContext=BB_AC061_W,ManagedElement=BB_AC061_W,Equipment=1,FieldReplaceableUnit=RRU-6,RfPort=A 2581110032</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-09-18 08:00:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-18 16:25:49
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -432,7 +432,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-18 06:24:01</t>
+          <t>2026-09-18 10:51:36</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-18 06:24:01</t>
+          <t>2026-09-18 10:51:36</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,34 +578,34 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-18 07:13:07</t>
+          <t>2026-09-18 13:17:47</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-18 07:13:07</t>
+          <t>2026-09-18 13:17:47</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-18 14:03:04</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-18 14:03:04</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-18 14:48:32</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-18 14:48:32</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-18 08:41:39</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-18 08:41:39</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>DABOU_SODECI</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC932</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC932_W</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-18 10:03:48</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-18 10:03:48</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2577806954</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-15 11:10:57</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,54 +1047,54 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-18 06:57:02</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-18 06:57:02</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,34 +1104,34 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-15 11:10:57</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2579832121</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,24 +1449,24 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-17 22:09:40</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,57 +1516,54 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1576,67 +1573,64 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>245</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1646,67 +1640,64 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-17 22:09:40</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1716,34 +1707,34 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1753,7 +1744,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1762,7 +1753,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>31</v>
+        <v>250</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1771,12 +1762,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1786,7 +1777,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1796,7 +1787,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -1808,12 +1799,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1823,7 +1814,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1832,21 +1823,21 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>20</v>
+        <v>245</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-18 07:57:51</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-18 07:57:51</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1856,7 +1847,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=356, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1866,40 +1857,43 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>31</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1908,12 +1902,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1923,64 +1917,67 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>31</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-18 06:14:08</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-18 06:14:08</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1990,64 +1987,67 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>20</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-18 06:15:23</t>
+          <t>2026-09-18 09:11:51</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-18 06:15:23</t>
+          <t>2026-09-18 09:11:51</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2057,64 +2057,64 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=353, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-18 06:16:43</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-18 06:16:43</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2156,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2176,12 +2176,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-18 06:22:29</t>
+          <t>2026-09-18 06:14:08</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-18 06:22:29</t>
+          <t>2026-09-18 06:14:08</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -2213,12 +2213,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2228,27 +2228,27 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-18 06:15:23</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-18 06:15:23</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -2280,42 +2280,42 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-18 06:16:43</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-18 06:16:43</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -2347,12 +2347,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2362,27 +2362,27 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-18 06:22:29</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-18 06:22:29</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,24 +2402,24 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2481,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2511,12 +2511,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-18 05:28:49</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-18 07:15:14</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
@@ -2548,12 +2548,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2578,12 +2578,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-18 06:36:18</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-18 07:29:42</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,24 +2603,24 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-18 06:43:00</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-18 07:37:45</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,34 +2670,34 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-18 06:47:49</t>
+          <t>2026-09-18 15:10:25</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-18 07:45:04</t>
+          <t>2026-09-18 15:10:25</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,57 +2737,54 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-18 15:40:21</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-18 15:40:21</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2797,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2807,57 +2804,54 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>KM4</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC098</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>LAC098</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>1.8</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-09-18 15:49:26</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-09-18 15:49:26</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2867,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC098,ManagedElement=1,TransportNetwork=1,Synchronization=1 2579063722</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2877,24 +2871,24 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>AKRIDOU_LASSE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>ET150</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2904,30 +2898,27 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>WET150</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>2.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-18 15:52:31</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-18 15:52:31</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2937,7 +2928,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET150,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581004188</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2947,57 +2938,54 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>GBAGBAM</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC790</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>WAC790</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-18 15:52:32</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-18 15:52:32</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3007,7 +2995,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC790,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576224038</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3017,57 +3005,54 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>GD_BEREBY</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC160</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>LAC160</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-18 15:52:40</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-18 15:52:40</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3077,7 +3062,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC160,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581313405</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3087,57 +3072,54 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>KOTIESSOU</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>AC763</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>AC763-OSmon</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>11.6</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-15 12:26:40</t>
+          <t>1970-01-09 21:31:22</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-15 12:26:40</t>
+          <t>1970-01-09 21:32:46</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3147,7 +3129,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2581313404</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3157,57 +3139,54 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TRANSUA</t>
+          <t>KOTIESSOU</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC566</t>
+          <t>AC763</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BB_AC566_W</t>
+          <t>AC763-OSmon</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>1.9</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-18 00:08:08</t>
+          <t>1970-01-09 21:32:46</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-18 00:08:08</t>
+          <t>1970-01-09 21:32:46</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3217,7 +3196,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2581317322</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3227,34 +3206,34 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>DJIBI</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AC061</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BB_AC061_W</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3272,12 +3251,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-18 06:37:09</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-18 06:37:09</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3287,7 +3266,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,MeContext=BB_AC061_W,ManagedElement=BB_AC061_W,Equipment=1,FieldReplaceableUnit=RRU-6,RfPort=A 2581110032</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3297,7 +3276,707 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-18 08:00:06</t>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ADAOU</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AC548</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BB_AC548_W</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>KOUWEIT_PIERRE_GADIE</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ET425</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BB_ET425_GL</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-09-15 12:26:40</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-09-15 12:26:40</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ABENGOUROU</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TRANSUA</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AC566</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BB_AC566_W</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-09-18 00:08:08</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-09-18 00:08:08</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>JACQUEVIL</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>AC211</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BB_AC211_GL</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:12:38</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:12:38</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>5</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SONGON_BEL_HORIZON</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ET815</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BB_ET815_GL</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:30:37</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:30:37</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2578625791</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:17:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-19 16:32:42
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-19 05:51:33</t>
+          <t>2026-09-19 08:46:29</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-19 05:51:33</t>
+          <t>2026-09-19 08:46:29</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-19 07:52:46</t>
+          <t>2026-09-19 11:11:13</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-19 07:52:46</t>
+          <t>2026-09-19 11:11:13</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,24 +645,24 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-19 07:54:46</t>
+          <t>2026-09-19 12:10:21</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-19 07:54:46</t>
+          <t>2026-09-19 12:10:21</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -712,39 +712,39 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-19 07:36:05</t>
+          <t>2026-09-19 13:51:41</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-19 07:36:05</t>
+          <t>2026-09-19 13:51:41</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-19 12:54:45</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-19 12:54:45</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,24 +1047,24 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,54 +1114,54 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-19 07:27:08</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-19 07:27:08</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,17 +1171,17 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -1908,12 +1908,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-18 09:11:51</t>
+          <t>2026-09-19 15:55:51</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-18 09:11:51</t>
+          <t>2026-09-19 15:55:51</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=353, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=357, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2548,22 +2548,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>TANRY</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC157</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC157</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2578,12 +2578,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-19 07:32:00</t>
+          <t>2026-09-19 14:28:51</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-19 07:32:00</t>
+          <t>2026-09-19 14:28:51</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC157,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581693029</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,24 +2603,24 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>HERMANKONO_DIES</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC772</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC772</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-19 07:33:48</t>
+          <t>2026-09-19 14:57:43</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-19 07:33:48</t>
+          <t>2026-09-19 15:56:42</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC772,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576053558</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-19 07:34:25</t>
+          <t>2026-09-19 14:57:45</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-19 07:34:25</t>
+          <t>2026-09-19 15:56:41</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581010108</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
@@ -2749,45 +2749,42 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>AKRIDOU_LASSE</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>ET150</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>WET150</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-19 14:57:46</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-19 15:53:27</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2797,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET150,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581004188</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2807,57 +2804,54 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>NIAMBEZARIA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET196</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>WET196</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>1.8</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-09-19 14:57:48</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-09-19 15:57:20</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2867,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET196,ManagedElement=1,TransportNetwork=1,Synchronization=1 2580997386</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2877,24 +2871,24 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>ADEBEM</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>ET287</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2904,30 +2898,27 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>WET287</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>2.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-19 14:57:55</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-19 15:56:42</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2937,7 +2928,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET287,ManagedElement=1,TransportNetwork=1,Synchronization=1 2580997004</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2947,57 +2938,54 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>KOTCHERI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>ET151</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>WET151</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-19 14:57:59</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-19 15:56:35</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3007,7 +2995,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET151,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576384110</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3017,57 +3005,54 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>NONOUAN</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC760</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>WAC760</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-19 14:58:11</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-19 15:57:19</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3077,7 +3062,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581697449</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3087,57 +3072,54 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TRANSUA</t>
+          <t>NONOUAN</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC566</t>
+          <t>AC760</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_AC566_W</t>
+          <t>LAC760</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>1.9</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-18 00:08:08</t>
+          <t>2026-09-19 14:59:34</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-18 00:08:08</t>
+          <t>2026-09-19 15:56:54</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3147,7 +3129,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581664159</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3157,57 +3139,54 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>IBOKE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>AC819</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>LAC819</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>5</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-09-19 15:00:14</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-09-19 15:53:27</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3217,7 +3196,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC819,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581692969</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3227,57 +3206,54 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>SASSANDRA_PHARE</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>ET371</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>WET371</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>4.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-19 15:01:39</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-19 15:56:46</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3287,7 +3263,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET371,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581635948</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3297,57 +3273,54 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>SOTREF</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>AC152</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>WAC152</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>4.5</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-18 19:59:53</t>
+          <t>2026-09-19 15:12:58</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-09-18 19:59:53</t>
+          <t>2026-09-19 15:12:58</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3357,7 +3330,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC152,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581699303</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3367,77 +3340,1846 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-19 07:59:52</t>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>GD_BEREBY</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AC160</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LAC160</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:13:21</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:13:21</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SubNetwork=EnodeB,MeContext=LAC160,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581313405</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SP_PLAGE</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ET370</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>WET370</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:13:21</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:13:21</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET370,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581694596</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ABENGOUROU</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>PANZAGANI</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ET440</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>WET440</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:15:07</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:15:07</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WET440,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581359907</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>DAKPADOU</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>AC767</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>WAC767</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:15:09</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:15:09</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>DJOUROUTOU</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AC787</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>WAC787</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:25:48</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:25:48</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>GBAPET</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>AC781</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LAC781</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:29:36</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:29:36</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>CANTONDOUGOU</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ET490</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>WET490</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:41:56</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:41:56</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET490,ManagedElement=1,TransportNetwork=1,Synchronization=1 2579316116</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>LOBAKUYA</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>AC773</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>WAC773</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:45:16</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:45:16</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC773,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581697446</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>CARR_ZEGBAN</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ET184</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>WET184</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:45:46</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:45:46</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET184,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581699349</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SASSANDRA</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>AC161</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>WAC161</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:47:32</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:47:32</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC161,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581694302</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SOGB_HEKE</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ET181</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>WET181</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:47:53</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:47:53</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET181,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581697447</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SASSANDRA_PHARE</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ET371</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LET371</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:48:11</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:48:11</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>SubNetwork=EnodeB,MeContext=LET371,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581695234</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>ABIDJAN 02</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>ASSOMPTION</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>ET017</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>BOUBOURY</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>AC534</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>BB_ET017_W</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>WAC534</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:51:22</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:51:22</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SAN-PEDRO</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PARA</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ET178</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>WET178</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:56:33</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:56:33</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>GAGNOA</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>CHIEPO</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ET141</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>WET141</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:56:37</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-09-19 15:56:37</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WET141,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576334017</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>YAMOUSSOUKRO</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>KOTIESSOU</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>AC763</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>RAN</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>AC763-OSmon</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Temperature is near limits</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>1970-01-10 21:04:07</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>1970-01-10 21:04:32</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2581752349</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>YAMOUSSOUKRO</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>KOTIESSOU</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>AC763</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>RAN</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>AC763-OSmon</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Temperature is near limits</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>1970-01-10 21:04:32</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>1970-01-10 21:04:32</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2581754261</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>GAGNOA</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>GOUDI</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ET148</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>BB_ET148_GL</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G44" t="n">
+      <c r="G61" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-06-26 14:52:51</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ADAOU</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>AC548</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BB_AC548_W</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>KOUWEIT_PIERRE_GADIE</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>ET425</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>BB_ET425_GL</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ABENGOUROU</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>TRANSUA</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>AC566</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>BB_AC566_W</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-09-18 00:08:08</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2026-09-18 00:08:08</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>5</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>JACQUEVIL</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>AC211</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>BB_AC211_GL</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
         <v>1.5</v>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H69" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-09-19 07:39:51</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-09-19 07:39:51</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,MeContext=BB_ET017_W,ManagedElement=BB_ET017_W,Equipment=1,FieldReplaceableUnit=RRU-5,RfPort=B 2581522424</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2026-09-19 07:59:52</t>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:17:41</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:17:41</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>2026-09-19 16:17:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-20 00:07:03
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -578,39 +578,39 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-19 11:11:13</t>
+          <t>2026-09-19 12:54:45</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-19 11:11:13</t>
+          <t>2026-09-19 12:54:45</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,49 +635,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-19 12:10:21</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-19 12:10:21</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-19 13:51:41</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-19 13:51:41</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-19 12:54:45</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-19 12:54:45</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,54 +980,54 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-19 20:40:31</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-19 20:40:31</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,34 +1037,34 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-18 18:57:00</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,54 +1449,57 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>250</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,64 +1509,67 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>245</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-18 18:57:00</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,34 +1579,34 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1610,7 +1616,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1619,7 +1625,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>250</v>
+        <v>31</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1628,12 +1634,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-16 15:57:31</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1643,7 +1649,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1653,7 +1659,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1695,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>245</v>
+        <v>31</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1713,7 +1719,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1723,7 +1729,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -1735,12 +1741,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1750,7 +1756,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1759,21 +1765,21 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-19 20:41:52</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-19 20:41:52</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1783,7 +1789,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1793,43 +1799,40 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>31</v>
+          <t>RfPortReflectedPowerTooHigh</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1838,12 +1841,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1853,67 +1856,64 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>20</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-19 15:55:51</t>
+          <t>2026-09-19 06:53:47</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-19 15:55:51</t>
+          <t>2026-09-19 06:53:47</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1923,64 +1923,64 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=357, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-19 06:54:03</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-19 06:54:03</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2022,12 +2022,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2042,12 +2042,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-19 06:53:47</t>
+          <t>2026-09-19 06:55:44</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-19 06:53:47</t>
+          <t>2026-09-19 06:55:44</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2089,12 +2089,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2109,12 +2109,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-19 06:54:03</t>
+          <t>2026-09-19 06:57:01</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-19 06:54:03</t>
+          <t>2026-09-19 06:57:01</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2146,12 +2146,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2161,27 +2161,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-19 06:55:44</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-19 06:55:44</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2213,12 +2213,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2228,27 +2228,27 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-19 06:57:01</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-19 06:57:01</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2280,12 +2280,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2310,12 +2310,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,24 +2335,24 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2377,12 +2377,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2414,12 +2414,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-19 22:23:40</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-19 23:19:23</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,24 +2469,24 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>DAKPADOU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC767</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WAC767</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2511,12 +2511,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-09-19 22:38:14</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-19 23:30:12</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2548,12 +2548,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TANRY</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC157</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC157</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2578,12 +2578,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-19 14:28:51</t>
+          <t>2026-09-19 22:41:48</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-19 14:28:51</t>
+          <t>2026-09-19 23:36:13</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC157,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581693029</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,24 +2603,24 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HERMANKONO_DIES</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC772</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC772</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-19 14:57:43</t>
+          <t>2026-09-19 22:51:02</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-19 15:56:42</t>
+          <t>2026-09-19 23:44:36</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC772,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576053558</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2682,22 +2682,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-19 14:57:45</t>
+          <t>2026-09-19 23:55:10</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-19 15:56:41</t>
+          <t>2026-09-19 23:55:10</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581010108</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
@@ -2749,42 +2749,45 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>AKRIDOU_LASSE</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET150</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WET150</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1.6</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-19 14:57:46</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-19 15:53:27</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2797,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET150,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581004188</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,54 +2807,57 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>NIAMBEZARIA</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET196</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WET196</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>1.8</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-19 14:57:48</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-19 15:57:20</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2861,7 +2867,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET196,ManagedElement=1,TransportNetwork=1,Synchronization=1 2580997386</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2871,24 +2877,24 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ADEBEM</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ET287</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2898,27 +2904,30 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WET287</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>2.1</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-19 14:57:55</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-19 15:56:42</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2928,7 +2937,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET287,ManagedElement=1,TransportNetwork=1,Synchronization=1 2580997004</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2938,54 +2947,57 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KOTCHERI</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET151</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>WET151</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1.7</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-19 14:57:59</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-19 15:56:35</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2995,7 +3007,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET151,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576384110</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3005,54 +3017,57 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NONOUAN</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AC760</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>WAC760</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1.7</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-19 14:58:11</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-19 15:57:19</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3062,7 +3077,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581697449</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3072,54 +3087,57 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>NONOUAN</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC760</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>LAC760</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1.9</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-19 14:59:34</t>
+          <t>2026-09-18 00:08:08</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-19 15:56:54</t>
+          <t>2026-09-18 00:08:08</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3129,7 +3147,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581664159</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3139,54 +3157,57 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IBOKE</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC819</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>LAC819</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>5</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-19 15:00:14</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-19 15:53:27</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3196,7 +3217,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC819,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581692969</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3206,54 +3227,57 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SASSANDRA_PHARE</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ET371</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>WET371</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>4.1</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-19 15:01:39</t>
+          <t>2026-09-18 13:09:02</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-19 15:56:46</t>
+          <t>2026-09-18 13:09:02</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3263,7 +3287,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET371,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581635948</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3273,54 +3297,57 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SOTREF</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>AC152</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>WAC152</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>4.6</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-19 15:12:58</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-09-19 15:12:58</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3330,7 +3357,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC152,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581699303</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3340,1846 +3367,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>GD_BEREBY</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>AC160</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>4G</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>LAC160</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:13:21</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:13:21</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC160,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581313405</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>SP_PLAGE</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>ET370</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>WET370</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:13:21</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:13:21</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET370,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581694596</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>PANZAGANI</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>ET440</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>WET440</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:15:07</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:15:07</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WET440,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581359907</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>DAKPADOU</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>AC767</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>WAC767</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:15:09</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:15:09</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>DJOUROUTOU</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>AC787</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>WAC787</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:25:48</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:25:48</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>GBAPET</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>AC781</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>4G</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>LAC781</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:29:36</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:29:36</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>CANTONDOUGOU</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>ET490</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>WET490</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:41:56</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:41:56</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET490,ManagedElement=1,TransportNetwork=1,Synchronization=1 2579316116</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>LOBAKUYA</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>AC773</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>WAC773</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:45:16</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:45:16</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC773,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581697446</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>CARR_ZEGBAN</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>ET184</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>WET184</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:45:46</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:45:46</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET184,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581699349</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>SASSANDRA</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>AC161</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>WAC161</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:47:32</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:47:32</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC161,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581694302</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>SOGB_HEKE</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>ET181</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>WET181</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:47:53</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:47:53</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET181,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581697447</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>SASSANDRA_PHARE</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>ET371</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>4G</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>LET371</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:48:11</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:48:11</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>SubNetwork=EnodeB,MeContext=LET371,ManagedElement=1,TransportNetwork=1,Synchronization=1 2581695234</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>BOUBOURY</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>AC534</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>WAC534</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:51:22</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:51:22</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>SAN-PEDRO</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>PARA</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>ET178</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>WET178</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:56:33</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:56:33</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>GAGNOA</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>CHIEPO</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>ET141</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>WET141</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:56:37</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>2026-09-19 15:56:37</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WET141,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576334017</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>YAMOUSSOUKRO</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>KOTIESSOU</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>AC763</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>RAN</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>AC763-OSmon</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Temperature is near limits</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>1970-01-10 21:04:07</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>1970-01-10 21:04:32</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2581752349</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>YAMOUSSOUKRO</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>KOTIESSOU</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>AC763</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>RAN</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>AC763-OSmon</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Temperature is near limits</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>1970-01-10 21:04:32</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>1970-01-10 21:04:32</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2581754261</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>GAGNOA</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>GOUDI</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>ET148</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>BB_ET148_GL</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>2026-06-17 12:12:52</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>2026-06-17 12:12:52</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>2026-06-26 14:52:51</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>2026-06-26 14:52:51</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>ABIDJAN 01</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>ADAOU</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>AC548</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>BB_AC548_W</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>ET425</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>BB_ET425_GL</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G64" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G65" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>TRANSUA</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>AC566</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>BB_AC566_W</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G66" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>2026-09-18 00:08:08</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>2026-09-18 00:08:08</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
-        </is>
-      </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>GESCO</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>AC314</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>BB_AC314_GL</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G67" t="n">
-        <v>5</v>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>2026-09-18 10:35:17</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>2026-09-18 10:35:17</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>GESCO</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>AC314</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>BB_AC314_GL</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G68" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>2026-09-18 13:09:02</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>2026-09-18 13:09:02</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>JACQUEVIL</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>AC211</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>BB_AC211_GL</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G69" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:17:41</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:17:41</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>YOP_BAFOND</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>IM522</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>2G,3G</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>BB_IM522_GW</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G70" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:33:44</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:33:44</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>2026-09-19 16:17:58</t>
+          <t>2026-09-20 00:00:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-20 08:21:59
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-19 08:46:29</t>
+          <t>2026-09-20 04:07:50</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-19 08:46:29</t>
+          <t>2026-09-20 04:07:50</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,39 +578,39 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-19 12:54:45</t>
+          <t>2026-09-20 07:16:30</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-19 12:54:45</t>
+          <t>2026-09-20 07:16:30</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,49 +635,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-20 07:19:41</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-20 07:19:41</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-20 07:49:18</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-20 07:49:18</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-19 12:54:45</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-19 12:54:45</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,54 +980,54 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-19 20:40:31</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-19 20:40:31</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,34 +1037,34 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,54 +1181,54 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-20 07:41:31</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-20 07:41:31</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,17 +1238,17 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-18 18:57:00</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,57 +1449,54 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1509,67 +1506,64 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>245</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1579,67 +1573,64 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-18 18:57:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1649,34 +1640,34 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1686,7 +1677,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1695,7 +1686,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>31</v>
+        <v>250</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1704,12 +1695,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-16 15:57:31</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1719,7 +1710,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1729,7 +1720,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -1799,40 +1790,43 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>31</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1841,12 +1835,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1856,64 +1850,67 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>31</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-19 06:53:47</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-19 06:53:47</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1923,64 +1920,67 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>245</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-19 06:54:03</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-19 06:54:03</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1990,34 +1990,34 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2027,27 +2027,27 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-19 06:55:44</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-19 06:55:44</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2109,12 +2109,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-19 06:57:01</t>
+          <t>2026-09-20 06:45:54</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-19 06:57:01</t>
+          <t>2026-09-20 06:45:54</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2146,42 +2146,42 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-20 06:46:00</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-20 06:46:00</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2213,42 +2213,42 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>BB_ET191_GL</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-20 06:46:43</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-20 06:46:43</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2280,12 +2280,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>DJIRO_GNEPAHIO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>ET191</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2295,27 +2295,27 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BB_ET191_W</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-20 06:47:12</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-20 06:47:12</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,24 +2335,24 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2377,12 +2377,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2414,12 +2414,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-19 22:23:40</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-19 23:19:23</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2481,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DAKPADOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC767</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WAC767</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2511,12 +2511,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-19 22:38:14</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-19 23:30:12</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,24 +2536,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2578,12 +2578,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-19 22:41:48</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-19 23:36:13</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2645,12 +2645,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-19 22:51:02</t>
+          <t>2026-09-20 05:34:22</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-19 23:44:36</t>
+          <t>2026-09-20 07:16:39</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2682,22 +2682,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-19 23:55:10</t>
+          <t>2026-09-20 06:32:57</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-19 23:55:10</t>
+          <t>2026-09-20 07:27:22</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,57 +2737,54 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-20 07:35:02</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-20 07:35:02</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2797,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2807,57 +2804,54 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>1.8</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-09-20 07:39:46</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-26 14:52:51</t>
+          <t>2026-09-20 07:39:46</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2867,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2877,34 +2871,34 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2913,7 +2907,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>2.1</v>
+        <v>1.6</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2922,12 +2916,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2937,7 +2931,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2947,7 +2941,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -2959,12 +2953,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2974,7 +2968,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2983,7 +2977,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2992,12 +2986,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-06-26 14:52:51</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3007,7 +3001,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2561805571</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3017,34 +3011,34 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3053,7 +3047,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -3062,12 +3056,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3077,7 +3071,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3087,34 +3081,34 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TRANSUA</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC566</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_AC566_W</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3123,7 +3117,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -3132,12 +3126,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-18 00:08:08</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-18 00:08:08</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3147,7 +3141,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3157,7 +3151,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -3169,12 +3163,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3184,7 +3178,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3193,7 +3187,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>5</v>
+        <v>1.7</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -3202,12 +3196,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3217,7 +3211,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3227,7 +3221,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -3263,7 +3257,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -3272,12 +3266,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3287,7 +3281,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3297,7 +3291,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-20 00:00:01</t>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>
@@ -3309,65 +3303,205 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-20 07:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>YOP_BAFOND</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>IM522</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>2G,3G</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>BB_IM522_GW</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G43" t="n">
+      <c r="G44" t="n">
         <v>4.6</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>2026-09-19 11:33:44</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>2026-09-19 11:33:44</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>ERICSSON</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-09-20 00:00:01</t>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-20 07:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ABENGOUROU</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TRANSUA</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AC566</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BB_AC566_W</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-09-20 04:57:39</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-09-20 04:57:39</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-20 07:59:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-20 16:39:44
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,10 +424,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-20 04:07:50</t>
+          <t>2026-09-20 11:56:50</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-20 04:07:50</t>
+          <t>2026-09-20 11:56:50</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -578,34 +578,34 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-20 07:16:30</t>
+          <t>2026-09-20 12:53:19</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-20 07:16:30</t>
+          <t>2026-09-20 12:53:19</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,24 +645,24 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-20 07:19:41</t>
+          <t>2026-09-20 14:38:39</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-20 07:19:41</t>
+          <t>2026-09-20 14:38:39</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -712,39 +712,39 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-20 07:49:18</t>
+          <t>2026-09-19 12:54:45</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-20 07:49:18</t>
+          <t>2026-09-19 12:54:45</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,17 +769,17 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>DABOU_SODECI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC932</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_AC932_W</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-19 12:54:45</t>
+          <t>2026-09-20 10:38:32</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-19 12:54:45</t>
+          <t>2026-09-20 10:38:32</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2582011075</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>BEKOUKOUIFIN</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>ET337</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_ET337_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Taken Out of Service</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-09-20 13:35:58</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-20 15:37:10</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,24 +1047,24 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,54 +1181,54 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-20 07:41:31</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-20 07:41:31</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,17 +1238,17 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-18 18:57:00</t>
+          <t>2026-09-20 10:53:47</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1732,12 +1732,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1756,21 +1756,21 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-19 20:41:52</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-19 20:41:52</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>31</v>
+        <v>245</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -1942,12 +1942,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1966,21 +1966,21 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>245</v>
+        <v>20</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-20 07:23:37</t>
+          <t>2026-09-20 15:29:52</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-20 07:23:37</t>
+          <t>2026-09-20 15:29:52</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=355, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2603,24 +2603,24 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-20 05:34:22</t>
+          <t>2026-09-20 14:34:12</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-20 07:16:39</t>
+          <t>2026-09-20 15:28:08</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-20 06:32:57</t>
+          <t>2026-09-20 15:27:04</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-20 07:27:22</t>
+          <t>2026-09-20 15:27:04</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2749,22 +2749,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2779,12 +2779,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-20 07:35:02</t>
+          <t>2026-09-20 15:47:24</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-20 07:35:02</t>
+          <t>2026-09-20 15:47:24</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2826,12 +2826,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2846,12 +2846,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-20 07:39:46</t>
+          <t>2026-09-20 15:55:10</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-20 07:39:46</t>
+          <t>2026-09-20 15:55:10</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>
@@ -3476,12 +3476,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-09-20 04:57:39</t>
+          <t>2026-09-20 11:08:50</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-09-20 04:57:39</t>
+          <t>2026-09-20 11:08:50</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3501,7 +3501,77 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-09-20 07:59:38</t>
+          <t>2026-09-20 16:18:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>JACQUEVIL</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>AC211</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BB_AC211_GL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-09-20 11:48:42</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-09-20 11:48:42</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-20 16:18:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-21 00:35:33
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -427,7 +427,7 @@
   <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:56:50</t>
+          <t>2026-09-20 17:57:36</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:56:50</t>
+          <t>2026-09-20 17:57:36</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,34 +578,34 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-20 12:53:19</t>
+          <t>2026-09-20 23:42:06</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-20 12:53:19</t>
+          <t>2026-09-20 23:42:06</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-20 14:38:39</t>
+          <t>2026-09-20 22:21:19</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-20 14:38:39</t>
+          <t>2026-09-20 22:21:19</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>BEKOUKOUIFIN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>ET337</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_ET337_GL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Critical Temperature Taken Out of Service</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-19 12:54:45</t>
+          <t>2026-09-20 23:56:52</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-19 12:54:45</t>
+          <t>2026-09-20 23:56:52</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -779,39 +779,39 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DABOU_SODECI</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC932</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_AC932_W</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-20 10:38:32</t>
+          <t>2026-07-22 20:53:20</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-20 10:38:32</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2582011075</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BEKOUKOUIFIN</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ET337</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_ET337_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Critical Temperature Taken Out of Service</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-20 13:35:58</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-20 15:37:10</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-07-22 20:53:20</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -1059,12 +1059,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,54 +1114,54 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-20 23:42:39</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-20 23:42:39</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,34 +1171,34 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -1461,12 +1461,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,24 +1516,24 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,54 +1583,57 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>250</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-20 10:53:47</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,34 +1643,34 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1677,7 +1680,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1686,7 +1689,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>250</v>
+        <v>31</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1695,12 +1698,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-20 07:23:37</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1710,7 +1713,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1720,7 +1723,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1783,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1790,7 +1793,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1829,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>31</v>
+        <v>245</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1850,7 +1853,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1860,7 +1863,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -1872,12 +1875,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1887,7 +1890,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1896,21 +1899,21 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>245</v>
+        <v>20</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-20 07:23:37</t>
+          <t>2026-09-20 21:09:52</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-20 07:23:37</t>
+          <t>2026-09-20 21:09:52</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1920,7 +1923,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=363, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1930,24 +1933,24 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BOUNANTINFLA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET734</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1957,7 +1960,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BOUNANTINFLA</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1975,12 +1978,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-20 15:29:52</t>
+          <t>2026-09-20 23:56:32</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-20 15:29:52</t>
+          <t>2026-09-20 23:56:32</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1990,7 +1993,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=355, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=349, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2000,7 +2003,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2070,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2137,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2204,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2271,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2338,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2405,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2472,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2539,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2603,24 +2606,24 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2630,7 +2633,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2645,12 +2648,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-20 14:34:12</t>
+          <t>2026-09-20 22:07:48</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-20 15:28:08</t>
+          <t>2026-09-20 23:58:36</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2660,7 +2663,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2670,24 +2673,24 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2697,7 +2700,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2715,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-20 15:27:04</t>
+          <t>2026-09-20 23:12:53</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-20 15:27:04</t>
+          <t>2026-09-20 23:12:53</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2730,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,7 +2740,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2749,22 +2752,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2779,12 +2782,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-20 15:47:24</t>
+          <t>2026-09-20 23:18:18</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-20 15:47:24</t>
+          <t>2026-09-20 23:18:18</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2797,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,7 +2807,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2826,12 +2829,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2846,12 +2849,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-20 15:55:10</t>
+          <t>2026-09-20 23:20:01</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-20 15:55:10</t>
+          <t>2026-09-20 23:20:01</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2861,7 +2864,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2871,7 +2874,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2944,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3014,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3084,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3154,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3224,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3294,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3364,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3434,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3504,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>
@@ -3513,22 +3516,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>ASSOMPTION</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET017</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_ET017_W</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3546,12 +3549,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-09-20 11:48:42</t>
+          <t>2026-09-20 23:54:04</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-09-20 11:48:42</t>
+          <t>2026-09-20 23:54:04</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3561,7 +3564,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,MeContext=BB_ET017_W,ManagedElement=BB_ET017_W,Equipment=1,FieldReplaceableUnit=RRU-5,RfPort=B 2582236762</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -3571,7 +3574,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-09-20 16:18:11</t>
+          <t>2026-09-21 00:17:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-22 00:37:06
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -432,13 +432,13 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="208" customWidth="1" min="12" max="12"/>
+    <col width="204" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
@@ -518,27 +518,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-21 11:27:57</t>
+          <t>2026-09-21 14:11:27</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-21 11:27:57</t>
+          <t>2026-09-21 14:11:27</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-21 12:31:59</t>
+          <t>2026-09-21 17:31:14</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-21 12:31:59</t>
+          <t>2026-09-21 17:31:14</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=80/176, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-21 14:11:27</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-21 14:11:27</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-21 14:48:51</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-21 14:48:51</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-21 14:37:19</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-21 15:35:58</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
@@ -925,12 +925,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,54 +980,54 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-21 22:20:35</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-21 22:20:35</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,34 +1037,34 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,39 +1181,39 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TERMINAL_2</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ET903</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_ET903_WL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Indoor RAP Temperature Exceptional</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-21 15:59:07</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-21 15:59:07</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET903_WL,ManagedElement=BB_ET903_WL,Equipment=1,FieldReplaceableUnit=RD-1-3 2576221744</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,54 +1449,57 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>250</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,50 +1509,53 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>20</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1558,12 +1564,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,64 +1579,67 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>31</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,34 +1649,34 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1677,7 +1686,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1686,7 +1695,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>250</v>
+        <v>31</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1695,12 +1704,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1710,7 +1719,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1720,7 +1729,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
@@ -1756,11 +1765,11 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>20</v>
+        <v>245</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1780,7 +1789,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1790,7 +1799,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
@@ -1802,12 +1811,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1817,7 +1826,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1826,21 +1835,21 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-21 21:47:53</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-21 21:47:53</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1850,7 +1859,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=363, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1860,43 +1869,40 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>31</v>
+          <t>RfPortReflectedPowerTooHigh</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1905,12 +1911,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1920,53 +1926,50 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>245</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1975,12 +1978,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1990,67 +1993,64 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>20</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-21 15:55:53</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-21 15:55:53</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2060,34 +2060,34 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=350, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2097,12 +2097,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2112,12 +2112,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2137,24 +2137,24 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2164,27 +2164,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-21 06:41:46</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-21 06:41:46</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580681495</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
@@ -2216,42 +2216,42 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BB_ET191_W</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-21 06:42:12</t>
+          <t>2026-09-21 22:29:51</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-21 06:42:12</t>
+          <t>2026-09-21 23:29:36</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_RadioNode,MeContext=BB_ET191_W,ManagedElement=BB_ET191_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580668838</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
@@ -2283,42 +2283,42 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-21 12:05:44</t>
+          <t>2026-09-21 22:55:15</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-21 12:05:44</t>
+          <t>2026-09-21 23:51:15</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2580662849</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2338,54 +2338,54 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DJIRO_GNEPAHIO</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET191</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BB_ET191_GL</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-21 12:06:01</t>
+          <t>2026-09-21 23:13:41</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-21 12:06:01</t>
+          <t>2026-09-21 23:13:41</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET191_GL,ManagedElement=BB_ET191_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2580662850</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
@@ -2417,12 +2417,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-21 23:15:21</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-21 23:15:21</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2472,54 +2472,54 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>MARC_AKWABA2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET001</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>ET001-OSmon</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Temperature Outside Limits</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>1970-01-09 04:41:55</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>1970-01-09 04:42:03</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2582618264</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2539,54 +2539,57 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1.6</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2596,7 +2599,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2606,24 +2609,24 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2633,27 +2636,30 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>2.1</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2663,7 +2669,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2673,54 +2679,57 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1.7</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-21 14:51:55</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-21 15:45:34</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2730,7 +2739,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2740,54 +2749,57 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1.7</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-21 15:10:27</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-21 15:10:27</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2797,7 +2809,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2807,54 +2819,57 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>5</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-21 15:24:17</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-21 15:24:17</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2864,7 +2879,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2874,54 +2889,57 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KOTIESSOU</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC763</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AC763-OSmon</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>4.1</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1970-01-12 16:42:18</t>
+          <t>2026-09-18 13:09:02</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>1970-01-12 21:37:32</t>
+          <t>2026-09-18 13:09:02</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2931,7 +2949,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2582416993</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2941,54 +2959,57 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KOTIESSOU</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AC763</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AC763-OSmon</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>4.6</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1970-01-12 21:37:32</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>1970-01-12 21:37:32</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2998,7 +3019,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2582503232</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3008,34 +3029,34 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3044,7 +3065,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -3053,12 +3074,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-20 11:08:50</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-20 11:08:50</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3068,7 +3089,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3078,637 +3099,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>ABIDJAN 01</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>ADAOU</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>AC548</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>BB_AC548_W</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>2026-08-19 15:48:55</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>ET425</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>BB_ET425_GL</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>2026-09-08 21:18:56</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>GESCO</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>AC314</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>BB_AC314_GL</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>5</v>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-09-18 10:35:17</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2026-09-18 10:35:17</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>GESCO</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>AC314</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>BB_AC314_GL</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-09-18 13:09:02</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-09-18 13:09:02</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>YOP_BAFOND</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>IM522</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2G,3G</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>BB_IM522_GW</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:33:44</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:33:44</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>TRANSUA</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>AC566</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>BB_AC566_W</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-09-20 11:08:50</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2026-09-20 11:08:50</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>SONGON_BEL_HORIZON</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>ET815</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>BB_ET815_GL</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-09-21 15:15:30</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2026-09-21 15:15:30</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>JACQUEVIL</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>AC211</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>BB_AC211_GL</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-09-21 15:47:02</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>2026-09-21 15:47:02</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2576218165</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:17:56</t>
+          <t>2026-09-22 00:17:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-22 08:08:35
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -432,7 +432,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
@@ -523,12 +523,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-21 14:11:27</t>
+          <t>2026-09-21 17:31:14</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-21 14:11:27</t>
+          <t>2026-09-21 17:31:14</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-21 17:31:14</t>
+          <t>2026-09-22 07:47:41</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-21 17:31:14</t>
+          <t>2026-09-22 07:47:41</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-22 07:45:27</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-22 07:45:27</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -712,24 +712,24 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -779,24 +779,24 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,54 +980,54 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-21 22:20:35</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-21 22:20:35</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,64 +1037,64 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-21 22:20:35</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-21 22:20:35</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,17 +1104,17 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -1126,12 +1126,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,57 +1449,54 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1509,34 +1506,34 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1546,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1555,21 +1552,21 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1579,7 +1576,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1589,7 +1586,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -1625,11 +1622,11 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1649,7 +1646,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1659,7 +1656,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1716,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1729,7 +1726,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1762,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>245</v>
+        <v>31</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1789,7 +1786,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1799,7 +1796,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1808,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1826,7 +1823,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1835,21 +1832,21 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>20</v>
+        <v>245</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-21 21:47:53</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-21 21:47:53</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1859,7 +1856,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=363, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1869,54 +1866,57 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>20</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-22 07:09:53</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-22 07:09:53</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1926,64 +1926,67 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=374, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>ZEGA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET861</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>ZEGA</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>20</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-22 07:41:16</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-22 07:41:16</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1993,34 +1996,34 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>Cabinet No.=0, Subrack No.=91, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2030,12 +2033,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2045,12 +2048,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2060,7 +2063,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2070,7 +2073,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -2082,12 +2085,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2097,7 +2100,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2112,12 +2115,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2127,7 +2130,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2137,24 +2140,24 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2164,7 +2167,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2179,12 +2182,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2194,7 +2197,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2204,7 +2207,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -2216,22 +2219,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2246,12 +2249,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-21 22:29:51</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-21 23:29:36</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2261,7 +2264,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2271,24 +2274,24 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2298,7 +2301,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2313,12 +2316,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-21 22:55:15</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-21 23:51:15</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2328,7 +2331,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2338,24 +2341,24 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2365,7 +2368,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2380,12 +2383,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-21 23:13:41</t>
+          <t>2026-09-22 06:19:21</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-21 23:13:41</t>
+          <t>2026-09-22 07:18:55</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2395,7 +2398,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2405,7 +2408,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -2417,12 +2420,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2432,7 +2435,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2447,12 +2450,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-21 23:15:21</t>
+          <t>2026-09-22 06:52:12</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-21 23:15:21</t>
+          <t>2026-09-22 07:47:08</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2462,7 +2465,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2472,54 +2475,54 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MARC_AKWABA2</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ET001</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ET001-OSmon</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Temperature Outside Limits</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1970-01-09 04:41:55</t>
+          <t>2026-09-22 06:52:33</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>1970-01-09 04:42:03</t>
+          <t>2026-09-22 07:51:47</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2529,7 +2532,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2582618264</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2539,57 +2542,54 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G32" t="n">
-        <v>1.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-22 07:53:20</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-22 07:53:20</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -2621,45 +2621,42 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>KM4</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC098</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>LAC098</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>2.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-22 07:53:31</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-22 07:53:31</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2669,7 +2666,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC098,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582430212</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2679,57 +2676,54 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>MARC_AKWABA2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>ET001</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>ET001-OSmon</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>1.7</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>1970-01-09 09:25:48</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>1970-01-09 12:20:34</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2739,7 +2733,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2582641710</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2749,57 +2743,54 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>MARC_AKWABA2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET001</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>ET001-OSmon</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1.7</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>1970-01-09 12:20:34</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>1970-01-09 12:20:34</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2809,7 +2800,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2582680457</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2819,24 +2810,24 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2846,7 +2837,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2855,7 +2846,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>5</v>
+        <v>1.6</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2864,12 +2855,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2879,7 +2870,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2889,34 +2880,34 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2925,7 +2916,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>4.1</v>
+        <v>2.1</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2934,12 +2925,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2949,7 +2940,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2959,7 +2950,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
@@ -2971,22 +2962,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2995,7 +2986,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>4.6</v>
+        <v>1.7</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -3004,12 +2995,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3019,7 +3010,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3029,77 +3020,357 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-22 00:17:59</t>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:59:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>5</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:59:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:59:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:59:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>ABENGOUROU</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>TRANSUA</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>AC566</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>BB_AC566_W</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G39" t="n">
+      <c r="G43" t="n">
         <v>1.9</v>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>2026-09-20 11:08:50</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>2026-09-20 11:08:50</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>ERICSSON</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>2026-09-22 00:17:59</t>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:59:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-22 16:23:53
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,14 +424,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
@@ -523,12 +523,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-21 17:31:14</t>
+          <t>2026-09-22 11:29:22</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-21 17:31:14</t>
+          <t>2026-09-22 11:29:22</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-22 07:47:41</t>
+          <t>2026-09-22 13:42:13</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-22 07:47:41</t>
+          <t>2026-09-22 13:42:13</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-22 07:45:27</t>
+          <t>2026-09-22 14:41:06</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-22 07:45:27</t>
+          <t>2026-09-22 14:41:06</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-22 15:06:21</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-22 15:06:21</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-22 10:48:07</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-22 10:48:07</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -858,12 +858,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>BEKOUKOUIFIN</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET337</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET337_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Taken Out of Service</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-22 15:46:24</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-22 15:57:38</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -992,12 +992,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,54 +1047,54 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-21 22:20:35</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-21 22:20:35</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,34 +1104,34 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,24 +1181,24 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,24 +1449,24 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,57 +1516,54 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1576,53 +1573,50 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>20</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1631,12 +1625,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1646,67 +1640,64 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1716,34 +1707,34 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1753,7 +1744,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1762,7 +1753,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>31</v>
+        <v>250</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1771,12 +1762,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1786,7 +1777,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1796,7 +1787,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -1832,11 +1823,11 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>245</v>
+        <v>20</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1856,7 +1847,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1866,7 +1857,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -1878,12 +1869,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1893,7 +1884,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1902,21 +1893,21 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-22 07:09:53</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-22 07:09:53</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1926,7 +1917,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=374, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1936,24 +1927,24 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ZEGA</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET861</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1963,7 +1954,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ZEGA</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1972,21 +1963,21 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-22 07:41:16</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-22 07:41:16</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1996,7 +1987,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=91, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2006,40 +1997,43 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>245</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2048,12 +2042,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2063,64 +2057,67 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>20</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-22 15:09:53</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-22 15:09:53</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2130,34 +2127,34 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2167,12 +2164,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2182,12 +2179,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2197,7 +2194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2207,7 +2204,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2216,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2234,7 +2231,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2249,12 +2246,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2264,7 +2261,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2274,24 +2271,24 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2301,7 +2298,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2316,12 +2313,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2331,7 +2328,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2341,7 +2338,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -2353,12 +2350,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2368,7 +2365,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2383,12 +2380,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-22 06:19:21</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-22 07:18:55</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2398,7 +2395,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2408,24 +2405,24 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2435,7 +2432,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2450,12 +2447,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-22 06:52:12</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-22 07:47:08</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2465,7 +2462,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2475,7 +2472,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -2487,22 +2484,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>DAKPADOU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC767</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC767</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2517,12 +2514,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-22 06:52:33</t>
+          <t>2026-09-22 14:33:53</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-22 07:51:47</t>
+          <t>2026-09-22 15:32:05</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2532,7 +2529,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2542,7 +2539,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -2554,12 +2551,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>MATHIEUKRO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC269</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2569,7 +2566,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC269</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2584,12 +2581,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-22 07:53:20</t>
+          <t>2026-09-22 15:12:55</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-22 07:53:20</t>
+          <t>2026-09-22 15:12:55</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2599,7 +2596,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC269,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582833923</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2609,34 +2606,34 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>KM4</t>
+          <t>SOTREF</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC098</t>
+          <t>AC152</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>LAC098</t>
+          <t>WAC152</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2651,12 +2648,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-22 07:53:31</t>
+          <t>2026-09-22 15:37:04</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-22 07:53:31</t>
+          <t>2026-09-22 15:37:04</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2666,7 +2663,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC098,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582430212</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC152,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582868176</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2676,54 +2673,54 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MARC_AKWABA2</t>
+          <t>IBOKE</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ET001</t>
+          <t>AC819</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ET001-OSmon</t>
+          <t>WAC819</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1970-01-09 09:25:48</t>
+          <t>2026-09-22 15:49:13</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>1970-01-09 12:20:34</t>
+          <t>2026-09-22 15:49:13</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2733,7 +2730,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2582641710</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC819,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582735262</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2743,54 +2740,54 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MARC_AKWABA2</t>
+          <t>NERO_PALMCI</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET001</t>
+          <t>ET214</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ET001-OSmon</t>
+          <t>WET214</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>1970-01-09 12:20:34</t>
+          <t>2026-09-22 15:57:45</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>1970-01-09 12:20:34</t>
+          <t>2026-09-22 15:57:45</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2800,7 +2797,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2582680457</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET214,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582696069</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2810,57 +2807,54 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>KOTIESSOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC763</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>AC763-OSmon</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>1.6</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>1970-01-13 17:19:37</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>1970-01-13 20:17:51</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2870,7 +2864,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2582774545</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2880,57 +2874,54 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>KOTIESSOU</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC763</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>AC763-OSmon</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>2.1</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>1970-01-13 20:17:51</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>1970-01-13 20:17:51</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2940,7 +2931,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2582833498</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2950,43 +2941,40 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>GESTOCI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC094</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>IP</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>AC094PER6273_01</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>1.7</v>
+          <t>Transceiver Temperature High Warning</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2995,12 +2983,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-22 11:21:59</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-22 14:24:46</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3010,7 +2998,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=ROUTER,MeContext=AC094PER6273_01,ManagedElement=1,interfaces=1,interface=2/1 2576388604</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3020,24 +3008,24 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3047,7 +3035,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3056,7 +3044,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -3065,12 +3053,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3080,7 +3068,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3090,34 +3078,34 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3126,7 +3114,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>5</v>
+        <v>2.1</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -3135,12 +3123,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3150,7 +3138,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3160,7 +3148,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -3172,12 +3160,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3187,7 +3175,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3196,7 +3184,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>4.1</v>
+        <v>1.7</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -3205,12 +3193,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3220,7 +3208,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3230,7 +3218,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
@@ -3242,22 +3230,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3266,7 +3254,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>4.6</v>
+        <v>1.7</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -3275,12 +3263,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3290,7 +3278,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3300,77 +3288,357 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-22 07:59:52</t>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>5</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-22 16:18:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-22 16:18:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-22 16:18:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>ABENGOUROU</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>TRANSUA</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>AC566</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>BB_AC566_W</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G43" t="n">
+      <c r="G46" t="n">
         <v>1.9</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>2026-09-20 11:08:50</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>2026-09-20 11:08:50</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
         <is>
           <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>ERICSSON</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-09-22 07:59:52</t>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-22 16:18:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>SONGON_BEL_HORIZON</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ET815</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>BB_ET815_GL</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:23:21</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:23:21</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-22 16:18:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-23 00:17:05
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,14 +424,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-22 11:29:22</t>
+          <t>2026-09-22 20:58:47</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-22 11:29:22</t>
+          <t>2026-09-22 20:58:47</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-22 13:42:13</t>
+          <t>2026-09-22 21:49:44</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-22 13:42:13</t>
+          <t>2026-09-22 21:49:44</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,24 +645,24 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-22 14:41:06</t>
+          <t>2026-09-22 21:50:24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-22 14:41:06</t>
+          <t>2026-09-22 21:50:24</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -712,39 +712,39 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-22 15:06:21</t>
+          <t>2026-09-22 10:48:07</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-22 15:06:21</t>
+          <t>2026-09-22 10:48:07</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-22 10:48:07</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-22 10:48:07</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BEKOUKOUIFIN</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ET337</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_ET337_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Critical Temperature Taken Out of Service</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-22 15:46:24</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-22 15:57:38</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,24 +1047,24 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,54 +1181,54 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-22 20:08:58</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-22 20:08:58</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,34 +1238,34 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,24 +1449,24 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,24 +1583,24 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1650,54 +1650,57 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>250</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,34 +1710,34 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1744,7 +1747,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1753,21 +1756,21 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>250</v>
+        <v>20</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1777,7 +1780,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1787,7 +1790,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -1823,11 +1826,11 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1847,7 +1850,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1857,7 +1860,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1920,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1927,7 +1930,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1966,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>31</v>
+        <v>245</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1987,7 +1990,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1997,7 +2000,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2012,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2024,7 +2027,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2033,21 +2036,21 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>245</v>
+        <v>20</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-22 21:21:54</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-22 21:21:54</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2057,7 +2060,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=353, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2067,57 +2070,54 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>20</v>
+          <t>RfPortReflectedPowerTooHigh</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-22 15:09:53</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-22 15:09:53</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2127,34 +2127,34 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2164,12 +2164,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2179,12 +2179,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -2216,12 +2216,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2246,12 +2246,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -2283,12 +2283,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2313,12 +2313,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2338,24 +2338,24 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2380,12 +2380,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2405,24 +2405,24 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-09-22 22:20:34</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-22 23:15:08</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -2484,22 +2484,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DAKPADOU</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC767</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WAC767</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2514,12 +2514,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-22 14:33:53</t>
+          <t>2026-09-22 22:27:26</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-22 15:32:05</t>
+          <t>2026-09-22 23:20:28</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2539,24 +2539,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MATHIEUKRO</t>
+          <t>CHIEPO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC269</t>
+          <t>ET141</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC269</t>
+          <t>WET141</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2581,12 +2581,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-22 15:12:55</t>
+          <t>2026-09-22 23:13:25</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-22 15:12:55</t>
+          <t>2026-09-22 23:13:25</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC269,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582833923</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WET141,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576334017</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2606,54 +2606,57 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SOTREF</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC152</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC152</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>1.6</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-22 15:37:04</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-22 15:37:04</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2663,7 +2666,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC152,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582868176</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2673,24 +2676,24 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IBOKE</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC819</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2700,27 +2703,30 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC819</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>2.1</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-22 15:49:13</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-22 15:49:13</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2730,7 +2736,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC819,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582735262</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2740,54 +2746,57 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>NERO_PALMCI</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET214</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WET214</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1.7</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-22 15:57:45</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-22 15:57:45</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2797,7 +2806,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET214,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582696069</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2807,54 +2816,57 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>KOTIESSOU</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC763</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>AC763-OSmon</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>1.7</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>1970-01-13 17:19:37</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>1970-01-13 20:17:51</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2864,7 +2876,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2582774545</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2874,54 +2886,57 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KOTIESSOU</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC763</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>AC763-OSmon</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>5</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1970-01-13 20:17:51</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>1970-01-13 20:17:51</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2931,7 +2946,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2582833498</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2941,40 +2956,43 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GESTOCI</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AC094</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>IP</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AC094PER6273_01</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Transceiver Temperature High Warning</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>4.1</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2983,12 +3001,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-22 11:21:59</t>
+          <t>2026-09-18 13:09:02</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-22 14:24:46</t>
+          <t>2026-09-18 13:09:02</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2998,7 +3016,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=ROUTER,MeContext=AC094PER6273_01,ManagedElement=1,interfaces=1,interface=2/1 2576388604</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3008,34 +3026,34 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3044,7 +3062,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1.6</v>
+        <v>4.6</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -3053,12 +3071,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3068,7 +3086,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3078,24 +3096,24 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3105,7 +3123,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3114,7 +3132,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -3123,12 +3141,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-20 11:08:50</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-20 11:08:50</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3138,7 +3156,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3148,7 +3166,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>
@@ -3160,12 +3178,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>SONGON_BEL_HORIZON</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>ET815</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3175,7 +3193,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>BB_ET815_GL</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3184,7 +3202,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -3193,12 +3211,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-22 09:23:21</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-22 09:23:21</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3208,7 +3226,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3218,427 +3236,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-22 16:18:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>TIEVIESSOU</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>ET833</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>BB_ET833_GL</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2026-09-09 13:41:30</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>2026-09-22 16:18:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>GESCO</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>AC314</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>BB_AC314_GL</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>5</v>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-09-18 10:35:17</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2026-09-18 10:35:17</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-09-22 16:18:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>GESCO</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>AC314</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>BB_AC314_GL</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-09-18 13:09:02</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-09-18 13:09:02</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2026-09-22 16:18:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>YOP_BAFOND</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>IM522</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2G,3G</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>BB_IM522_GW</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:33:44</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:33:44</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>2026-09-22 16:18:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>TRANSUA</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>AC566</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>BB_AC566_W</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-09-20 11:08:50</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2026-09-20 11:08:50</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>2026-09-22 16:18:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>SONGON_BEL_HORIZON</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>ET815</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>BB_ET815_GL</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-09-22 09:23:21</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2026-09-22 09:23:21</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>2026-09-22 16:18:22</t>
+          <t>2026-09-23 00:00:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-23 08:08:31
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-22 21:49:44</t>
+          <t>2026-09-23 06:01:40</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-22 21:49:44</t>
+          <t>2026-09-23 06:01:40</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-22 21:50:24</t>
+          <t>2026-09-23 06:01:51</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-22 21:50:24</t>
+          <t>2026-09-23 06:01:51</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -779,24 +779,24 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>BEKOUKOUIFIN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>ET337</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -806,12 +806,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_ET337_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Taken Out of Service</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-23 07:20:31</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-23 07:50:28</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,24 +1047,24 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -1126,12 +1126,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,54 +1181,54 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-22 20:08:58</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-22 20:08:58</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,64 +1238,64 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-23 07:50:03</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-23 07:50:03</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,17 +1305,17 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,24 +1382,24 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,24 +1449,24 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,24 +1583,24 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1650,57 +1650,54 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1710,34 +1707,34 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1747,7 +1744,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1756,21 +1753,21 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1780,7 +1777,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1790,7 +1787,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -1826,11 +1823,11 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1850,7 +1847,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1860,7 +1857,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1917,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1930,7 +1927,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1963,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>245</v>
+        <v>31</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1990,7 +1987,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2000,7 +1997,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -2012,12 +2009,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2027,7 +2024,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2036,21 +2033,21 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>20</v>
+        <v>245</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-22 21:21:54</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-22 21:21:54</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2060,7 +2057,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=353, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2070,54 +2067,57 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>20</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-23 07:45:54</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-23 07:45:54</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2127,34 +2127,34 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=356, RF Port=NULL</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2164,12 +2164,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2179,12 +2179,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -2216,12 +2216,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2246,12 +2246,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -2283,12 +2283,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2313,12 +2313,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2338,24 +2338,24 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2380,12 +2380,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2405,24 +2405,24 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-22 22:20:34</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-22 23:15:08</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -2484,22 +2484,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2514,12 +2514,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-22 22:27:26</t>
+          <t>2026-09-23 05:37:02</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-22 23:20:28</t>
+          <t>2026-09-23 07:20:59</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2539,24 +2539,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CHIEPO</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ET141</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WET141</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2581,12 +2581,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-22 23:13:25</t>
+          <t>2026-09-23 06:29:40</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-22 23:13:25</t>
+          <t>2026-09-23 07:23:54</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WET141,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576334017</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2606,57 +2606,54 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>1.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-23 06:31:38</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-23 07:26:05</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2666,7 +2663,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2676,24 +2673,24 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2703,30 +2700,27 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>2.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-23 07:31:45</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-23 07:31:45</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2736,7 +2730,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2746,57 +2740,54 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>KAGBE</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC780</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>WAC780</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-23 07:52:24</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-23 07:52:24</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2806,7 +2797,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WAC780,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583083510</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2816,57 +2807,54 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>MARC_AKWABA2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET001</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>ET001-OSmon</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>1.7</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>1970-01-10 13:13:44</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>1970-01-10 13:45:45</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2876,7 +2864,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2583053811</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2886,57 +2874,54 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>MARC_AKWABA2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>ET001</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>ET001-OSmon</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>5</v>
+          <t>Temperature is near limits</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>1970-01-10 13:45:45</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>1970-01-10 13:45:45</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2946,7 +2931,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2583054049</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2956,24 +2941,24 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2983,7 +2968,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2992,7 +2977,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>4.1</v>
+        <v>1.6</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -3001,12 +2986,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3016,7 +3001,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3026,34 +3011,34 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3062,7 +3047,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>4.6</v>
+        <v>2.1</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -3071,12 +3056,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3086,7 +3071,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3096,34 +3081,34 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TRANSUA</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC566</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_AC566_W</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3132,7 +3117,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -3141,12 +3126,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-20 11:08:50</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-20 11:08:50</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3156,7 +3141,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3166,7 +3151,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-23 00:00:06</t>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>
@@ -3178,65 +3163,415 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:59:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>5</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:59:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:59:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:59:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>SONGON_BEL_HORIZON</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>ET815</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>2G,4G</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>BB_ET815_GL</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G41" t="n">
+      <c r="G45" t="n">
         <v>1.6</v>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>2026-09-22 09:23:21</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>2026-09-22 09:23:21</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>ERICSSON</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>2026-09-23 00:00:06</t>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:59:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ABENGOUROU</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TRANSUA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>AC566</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BB_AC566_W</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-09-23 03:35:57</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-09-23 03:35:57</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:59:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-23 16:36:13
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-22 20:58:47</t>
+          <t>2026-09-23 09:35:04</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-22 20:58:47</t>
+          <t>2026-09-23 09:35:04</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,24 +578,24 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-23 06:01:40</t>
+          <t>2026-09-23 09:37:09</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-23 06:01:40</t>
+          <t>2026-09-23 09:37:09</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,24 +645,24 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-23 06:01:51</t>
+          <t>2026-09-23 10:49:54</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-23 06:01:51</t>
+          <t>2026-09-23 10:49:54</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=0, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -712,39 +712,39 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-22 10:48:07</t>
+          <t>2026-09-23 13:50:53</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-22 10:48:07</t>
+          <t>2026-09-23 13:50:53</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BEKOUKOUIFIN</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET337</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET337_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical Temperature Taken Out of Service</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-23 07:20:31</t>
+          <t>2026-09-22 10:48:07</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-23 07:50:28</t>
+          <t>2026-09-22 10:48:07</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>DABOU_SODECI</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC932</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC932_W</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-23 12:23:55</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-23 12:23:55</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2583202212</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,24 +1047,24 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -1193,12 +1193,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,54 +1248,54 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-23 07:50:03</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-23 07:50:03</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,64 +1305,64 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Identity=Toggling Alarm, Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>ABOISSO_MUNICIPALITE</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>ET545</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>Microwave</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>ET545-ML6691</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temperature</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-23 09:52:02</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-23 09:52:02</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=MINILINK,MeContext=ET545-ML6691,ManagedElement=ET545-ML6691,NPU_1003=1/4 2582421010</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,24 +1449,24 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,24 +1516,24 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -1595,12 +1595,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1650,24 +1650,24 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1692,12 +1692,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1717,57 +1717,54 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1777,34 +1774,34 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1814,7 +1811,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1823,21 +1820,21 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1847,7 +1844,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1857,7 +1854,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -1893,11 +1890,11 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1917,7 +1914,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1927,7 +1924,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1984,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1997,7 +1994,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2030,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>245</v>
+        <v>31</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2057,7 +2054,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2067,7 +2064,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2079,12 +2076,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2094,7 +2091,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2103,21 +2100,21 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>20</v>
+        <v>245</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-23 07:45:54</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-23 07:45:54</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2127,7 +2124,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=356, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2137,7 +2134,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2201,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2268,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2335,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2402,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2472,24 +2469,24 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>PETIT_YAPO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>AC755</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2499,7 +2496,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>WAC755</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2514,12 +2511,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-23 05:37:02</t>
+          <t>2026-09-23 12:38:45</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-23 07:20:59</t>
+          <t>2026-09-23 12:38:45</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2529,7 +2526,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_GROUP,MeContext=WAC755,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583268253</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2539,7 +2536,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2551,12 +2548,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>TANRY</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC157</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2566,7 +2563,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC157</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2581,12 +2578,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-23 06:29:40</t>
+          <t>2026-09-23 14:03:34</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-23 07:23:54</t>
+          <t>2026-09-23 14:03:34</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2596,7 +2593,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC157,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582843199</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2606,7 +2603,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2618,22 +2615,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>DJOUROUTOU</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC787</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC787</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2648,12 +2645,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-23 06:31:38</t>
+          <t>2026-09-23 15:14:04</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-23 07:26:05</t>
+          <t>2026-09-23 15:14:04</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2663,7 +2660,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2673,34 +2670,34 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>KM4</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC098</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>LAC098</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2715,12 +2712,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-23 07:31:45</t>
+          <t>2026-09-23 15:21:18</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-23 07:31:45</t>
+          <t>2026-09-23 15:21:18</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2730,7 +2727,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC098,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582430212</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2740,7 +2737,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2752,12 +2749,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KAGBE</t>
+          <t>LAKOTA_NEW</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC780</t>
+          <t>AC966</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2767,7 +2764,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WAC780</t>
+          <t>WAC966</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2782,12 +2779,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-23 07:52:24</t>
+          <t>2026-09-23 15:21:50</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-23 07:52:24</t>
+          <t>2026-09-23 15:21:50</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2797,7 +2794,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WAC780,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583083510</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WAC966,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582998023</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2807,54 +2804,54 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MARC_AKWABA2</t>
+          <t>AGBO_MONTBLANC</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET001</t>
+          <t>ET339</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ET001-OSmon</t>
+          <t>WET339</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>1970-01-10 13:13:44</t>
+          <t>2026-09-23 15:21:51</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>1970-01-10 13:45:45</t>
+          <t>2026-09-23 15:21:51</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2864,7 +2861,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2583053811</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_GROUP,MeContext=WET339,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583014432</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2874,54 +2871,54 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MARC_AKWABA2</t>
+          <t>BIEBY</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ET001</t>
+          <t>AC749</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ET001-OSmon</t>
+          <t>WAC749</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1970-01-10 13:45:45</t>
+          <t>2026-09-23 15:21:51</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>1970-01-10 13:45:45</t>
+          <t>2026-09-23 15:21:51</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2931,7 +2928,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2583054049</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_GROUP,MeContext=WAC749,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582998022</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2941,7 +2938,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -2953,45 +2950,42 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>DJIDJIDOU</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>ET183</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>WET183</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>1.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-23 15:21:51</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-23 15:21:51</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3001,7 +2995,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WET183,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583022241</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3011,24 +3005,24 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>ANNO</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC744</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3038,30 +3032,27 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>WAC744</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>2.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-23 15:21:52</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-23 15:21:52</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3071,7 +3062,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_GROUP,MeContext=WAC744,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583022242</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3081,57 +3072,54 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>DIDOKO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC775</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>WAC775</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-23 15:21:53</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-23 15:21:53</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3141,7 +3129,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WAC775,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583237842</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3151,7 +3139,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
@@ -3163,45 +3151,42 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>1.7</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-23 15:22:11</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-23 15:22:11</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3211,7 +3196,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3221,57 +3206,54 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>HANNIE</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>ET187</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>WET187</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>5</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-09-23 15:22:36</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-09-23 15:22:36</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3281,7 +3263,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET187,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582843200</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3291,57 +3273,54 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>SASSANDRA_PHARE</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>ET371</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>LET371</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>4.1</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-23 15:22:40</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-23 15:22:40</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3351,7 +3330,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+          <t>SubNetwork=EnodeB,MeContext=LET371,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582774837</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3361,57 +3340,54 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>NONOUAN</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>AC760</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>WAC760</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>4.6</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-09-23 15:23:50</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-09-23 15:23:50</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3421,7 +3397,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582782842</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3431,57 +3407,54 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SONGON_BEL_HORIZON</t>
+          <t>MARC_AKWABA2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ET815</t>
+          <t>ET001</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BB_ET815_GL</t>
+          <t>ET001-OSmon</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>1.6</v>
+          <t>Temperature Outside Limits</t>
+        </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-09-22 09:23:21</t>
+          <t>1970-01-10 19:14:57</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-09-22 09:23:21</t>
+          <t>1970-01-10 19:15:15</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3491,7 +3464,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2583202806</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3501,77 +3474,908 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-09-23 07:59:36</t>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ANGRE_CIT</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ET084</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>RAN</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ET084-OSmon</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Temperature is near limits</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2007-02-07 14:02:30</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2007-02-07 14:02:30</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SubNetwork=TCU,MeContext=ET084-OSmon,STN=0,Equipment=0 2583229397</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>YAMOUSSOUKRO</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>KOTIESSOU</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>AC763</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>RAN</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>AC763-OSmon</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Temperature is near limits</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>1970-01-14 18:44:04</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>1970-01-14 21:33:34</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2583199817</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>YAMOUSSOUKRO</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>KOTIESSOU</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AC763</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>RAN</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>AC763-OSmon</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Temperature is near limits</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>1970-01-14 21:33:34</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>1970-01-14 21:33:34</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2583267549</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>GAGNOA</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>GOUDI</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ET148</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BB_ET148_GL</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:12:52</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ADAOU</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AC548</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>BB_AC548_W</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:48:55</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>KOUWEIT_PIERRE_GADIE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ET425</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BB_ET425_GL</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-08 21:18:56</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>BB_ET833_GL</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:41:30</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>5</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:35:17</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>GESCO</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>AC314</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>BB_AC314_GL</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:09:02</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>YOP_BAFOND</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>IM522</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2G,3G</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>BB_IM522_GW</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:33:44</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SONGON_BEL_HORIZON</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ET815</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>BB_ET815_GL</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:23:21</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:23:21</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>ABENGOUROU</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>TRANSUA</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>AC566</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>BB_AC566_W</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G46" t="n">
+      <c r="G57" t="n">
         <v>1.9</v>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>2026-09-23 03:35:57</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t>2026-09-23 03:35:57</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>2026-09-23 07:59:36</t>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>STAR_2</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>AC365</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>BB_AC365_GL</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:42:02</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:42:02</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC365_GL,ManagedElement=BB_AC365_GL,Equipment=1,FieldReplaceableUnit=RRUS-9_B3,RfPort=B 2583249128</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:15:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-24 10:24:17
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC203</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SINFRA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-23 09:35:04</t>
+          <t>2026-09-23 22:18:28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-23 09:35:04</t>
+          <t>2026-09-23 22:18:28</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,39 +578,39 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-23 09:37:09</t>
+          <t>2026-09-22 10:48:07</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-23 09:37:09</t>
+          <t>2026-09-22 10:48:07</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,49 +635,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BEKOUKOUIFIN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>ET337</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BB_ET337_GL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Taken Out of Service</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-23 10:49:54</t>
+          <t>2026-09-24 06:44:08</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-23 10:49:54</t>
+          <t>2026-09-24 07:54:42</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-23 13:50:53</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-23 13:50:53</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-22 10:48:07</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-22 10:48:07</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DABOU_SODECI</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC932</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC932_W</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-23 12:23:55</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-23 12:23:55</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2583202212</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,24 +913,24 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -992,12 +992,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,24 +1047,24 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,54 +1114,54 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-23 23:55:14</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-23 23:55:14</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,34 +1171,34 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,54 +1315,54 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ABOISSO_MUNICIPALITE</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ET545</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Microwave</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ET545-ML6691</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>High Temperature</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-23 09:52:02</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-23 09:52:02</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=MINILINK,MeContext=ET545-ML6691,ManagedElement=ET545-ML6691,NPU_1003=1/4 2582421010</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -1461,12 +1461,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,24 +1516,24 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,54 +1583,57 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>250</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-12 09:15:07</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,50 +1643,53 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>20</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1692,12 +1698,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,64 +1713,67 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>31</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1774,34 +1783,34 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1811,7 +1820,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1820,7 +1829,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>250</v>
+        <v>31</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1829,12 +1838,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1844,7 +1853,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1854,7 +1863,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -1890,11 +1899,11 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>20</v>
+        <v>245</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1914,7 +1923,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1924,7 +1933,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -1936,12 +1945,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1951,7 +1960,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1960,21 +1969,21 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-23 20:55:54</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-23 20:55:54</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1984,7 +1993,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=351, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1994,43 +2003,40 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>31</v>
+          <t>RfPortReflectedPowerTooHigh</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2039,12 +2045,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2054,53 +2060,50 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>245</v>
+          <t>Sync Reference PDV Problem</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2109,12 +2112,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2124,34 +2127,34 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2161,12 +2164,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2176,12 +2179,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2191,7 +2194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2201,7 +2204,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -2213,12 +2216,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2228,7 +2231,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2243,12 +2246,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,7 +2261,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2268,24 +2271,24 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2295,7 +2298,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2310,12 +2313,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2325,7 +2328,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2335,24 +2338,24 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>BONDOUKOU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC182</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2362,7 +2365,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>WAC182</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2377,12 +2380,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-24 04:28:23</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-24 04:28:23</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2392,7 +2395,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC182,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583505337</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2402,24 +2405,24 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2429,7 +2432,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2444,12 +2447,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-09-24 06:21:35</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-24 07:18:57</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2459,7 +2462,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2469,34 +2472,34 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PETIT_YAPO</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC755</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WAC755</t>
+          <t>LAC781</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2511,12 +2514,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-23 12:38:45</t>
+          <t>2026-09-24 06:30:28</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-23 12:38:45</t>
+          <t>2026-09-24 07:21:57</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2526,7 +2529,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_GROUP,MeContext=WAC755,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583268253</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2536,24 +2539,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TANRY</t>
+          <t>KAMAGAYA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC157</t>
+          <t>AC731</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2563,7 +2566,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC157</t>
+          <t>WAC731</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2578,12 +2581,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-23 14:03:34</t>
+          <t>2026-09-24 07:36:55</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-23 14:03:34</t>
+          <t>2026-09-24 07:36:55</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2593,7 +2596,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC157,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582843199</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC731,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583487709</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2603,7 +2606,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -2645,12 +2648,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-23 15:14:04</t>
+          <t>2026-09-24 07:40:17</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-23 15:14:04</t>
+          <t>2026-09-24 07:40:17</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2670,34 +2673,34 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>KM4</t>
+          <t>GBAPET</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC098</t>
+          <t>AC781</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>LAC098</t>
+          <t>WAC781</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2712,12 +2715,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:18</t>
+          <t>2026-09-24 07:41:29</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:18</t>
+          <t>2026-09-24 07:41:29</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2727,7 +2730,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC098,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582430212</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2737,24 +2740,24 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>LAKOTA_NEW</t>
+          <t>KROKROM</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC966</t>
+          <t>AC221</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2764,7 +2767,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WAC966</t>
+          <t>WAC221</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2779,12 +2782,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:50</t>
+          <t>2026-09-24 07:47:13</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:50</t>
+          <t>2026-09-24 07:47:13</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2794,7 +2797,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WAC966,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582998023</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC221,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582833603</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2804,24 +2807,24 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AGBO_MONTBLANC</t>
+          <t>DAKPADOU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ET339</t>
+          <t>AC767</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2831,7 +2834,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WET339</t>
+          <t>WAC767</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2846,12 +2849,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:51</t>
+          <t>2026-09-24 07:47:14</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:51</t>
+          <t>2026-09-24 07:47:14</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2861,7 +2864,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_GROUP,MeContext=WET339,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583014432</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2871,24 +2874,24 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BIEBY</t>
+          <t>SASSANDRA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC749</t>
+          <t>AC161</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2898,7 +2901,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WAC749</t>
+          <t>WAC161</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2913,12 +2916,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:51</t>
+          <t>2026-09-24 07:47:22</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:51</t>
+          <t>2026-09-24 07:47:22</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2928,7 +2931,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_GROUP,MeContext=WAC749,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582998022</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC161,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583331220</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2938,7 +2941,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -2950,12 +2953,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DJIDJIDOU</t>
+          <t>NIAMBEZARIA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET183</t>
+          <t>ET196</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2965,7 +2968,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>WET183</t>
+          <t>WET196</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2980,12 +2983,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:51</t>
+          <t>2026-09-24 07:47:24</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:51</t>
+          <t>2026-09-24 07:47:24</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2995,7 +2998,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WET183,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583022241</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET196,ManagedElement=1,TransportNetwork=1,Synchronization=1 2580997386</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3005,24 +3008,24 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ANNO</t>
+          <t>KOTCHERI</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AC744</t>
+          <t>ET151</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3032,7 +3035,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>WAC744</t>
+          <t>WET151</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3047,12 +3050,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:52</t>
+          <t>2026-09-24 07:47:28</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:52</t>
+          <t>2026-09-24 07:47:28</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3062,7 +3065,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_GROUP,MeContext=WAC744,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583022242</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET151,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576384110</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3072,24 +3075,24 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>DIDOKO</t>
+          <t>CANTONDOUGOU</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AC775</t>
+          <t>ET490</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3099,7 +3102,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>WAC775</t>
+          <t>WET490</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3114,12 +3117,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:53</t>
+          <t>2026-09-24 07:47:28</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-23 15:21:53</t>
+          <t>2026-09-24 07:47:28</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3129,7 +3132,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WAC775,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583237842</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET490,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582774827</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3139,24 +3142,24 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>CHIEPO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET141</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3166,7 +3169,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>WET141</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3181,12 +3184,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-23 15:22:11</t>
+          <t>2026-09-24 07:47:30</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-23 15:22:11</t>
+          <t>2026-09-24 07:47:30</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3196,7 +3199,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576168106</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WET141,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576334017</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3206,7 +3209,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3221,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>HANNIE</t>
+          <t>NONOUAN</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ET187</t>
+          <t>AC760</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3233,7 +3236,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>WET187</t>
+          <t>WAC760</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3248,12 +3251,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-23 15:22:36</t>
+          <t>2026-09-24 07:47:34</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-23 15:22:36</t>
+          <t>2026-09-24 07:47:34</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3263,7 +3266,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET187,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582843200</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582782842</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3273,7 +3276,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -3315,12 +3318,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-23 15:22:40</t>
+          <t>2026-09-24 07:47:43</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-09-23 15:22:40</t>
+          <t>2026-09-24 07:47:43</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3340,7 +3343,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -3362,12 +3365,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>WAC760</t>
+          <t>LAC760</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3382,12 +3385,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-09-23 15:23:50</t>
+          <t>2026-09-24 07:48:07</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-09-23 15:23:50</t>
+          <t>2026-09-24 07:48:07</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3397,7 +3400,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582782842</t>
+          <t>SubNetwork=EnodeB,MeContext=LAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583487821</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3407,54 +3410,54 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MARC_AKWABA2</t>
+          <t>NERO_PALMCI</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ET001</t>
+          <t>ET214</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ET001-OSmon</t>
+          <t>WET214</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Temperature Outside Limits</t>
+          <t>Sync Reference PDV Problem</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>1970-01-10 19:14:57</t>
+          <t>2026-09-24 07:48:21</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>1970-01-10 19:15:15</t>
+          <t>2026-09-24 07:48:21</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3464,7 +3467,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2583202806</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET214,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583505436</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3474,54 +3477,57 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ANGRE_CIT</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ET084</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ET084-OSmon</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1.6</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2007-02-07 14:02:30</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2007-02-07 14:02:30</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3531,7 +3537,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=ET084-OSmon,STN=0,Equipment=0 2583229397</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -3541,54 +3547,57 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>KOTIESSOU</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>AC763</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>AC763-OSmon</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>2.1</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>1970-01-14 18:44:04</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>1970-01-14 21:33:34</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3598,7 +3607,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2583199817</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3608,54 +3617,57 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>KOTIESSOU</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AC763</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>AC763-OSmon</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Temperature is near limits</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1.7</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>1970-01-14 21:33:34</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>1970-01-14 21:33:34</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3665,7 +3677,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC763-OSmon,STN=0,Equipment=0 2583267549</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3675,24 +3687,24 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3702,7 +3714,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3711,7 +3723,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3720,12 +3732,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3735,7 +3747,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3745,34 +3757,34 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3781,7 +3793,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>2.1</v>
+        <v>5</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -3790,12 +3802,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-18 10:35:17</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-24 07:36:44</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3805,7 +3817,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -3815,7 +3827,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -3827,22 +3839,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3851,7 +3863,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>1.7</v>
+        <v>4.6</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -3860,12 +3872,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3875,7 +3887,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -3885,7 +3897,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
@@ -3897,12 +3909,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>SONGON_BEL_HORIZON</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET815</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3912,7 +3924,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_ET815_GL</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3921,7 +3933,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -3930,12 +3942,12 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-22 09:23:21</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-22 09:23:21</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3945,7 +3957,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -3955,34 +3967,34 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3991,7 +4003,7 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>5</v>
+        <v>1.9</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -4000,12 +4012,12 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-09-23 03:35:57</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-09-18 10:35:17</t>
+          <t>2026-09-23 03:35:57</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4015,7 +4027,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -4025,24 +4037,24 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>GESCO</t>
+          <t>STAR_2</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>AC314</t>
+          <t>AC365</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -4052,7 +4064,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>BB_AC314_GL</t>
+          <t>BB_AC365_GL</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4061,7 +4073,7 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>4.1</v>
+        <v>3.3</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -4070,12 +4082,12 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-23 14:42:02</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-09-18 13:09:02</t>
+          <t>2026-09-23 14:42:02</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -4085,7 +4097,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC365_GL,ManagedElement=BB_AC365_GL,Equipment=1,FieldReplaceableUnit=RRUS-9_B3,RfPort=B 2583249128</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -4095,34 +4107,34 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YOP_BAFOND</t>
+          <t>YAKASSE_ME</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>IM522</t>
+          <t>AC543</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2G,3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>BB_IM522_GW</t>
+          <t>BB_AC543_GL</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4131,7 +4143,7 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>4.6</v>
+        <v>5.8</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -4140,12 +4152,12 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-09-24 07:04:03</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-09-19 11:33:44</t>
+          <t>2026-09-24 07:04:03</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -4155,7 +4167,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC543_GL,ManagedElement=BB_AC543_GL,Equipment=1,FieldReplaceableUnit=RRUS-7_B1B3,RfPort=D 2583350904</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -4165,217 +4177,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>2026-09-23 16:15:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>SONGON_BEL_HORIZON</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>ET815</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>BB_ET815_GL</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>2026-09-22 09:23:21</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>2026-09-22 09:23:21</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>2026-09-23 16:15:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>TRANSUA</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>AC566</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>BB_AC566_W</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>2026-09-23 03:35:57</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>2026-09-23 03:35:57</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>2026-09-23 16:15:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>ABIDJAN 03</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>STAR_2</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>AC365</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>BB_AC365_GL</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G58" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>2026-09-23 14:42:02</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>2026-09-23 14:42:02</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC365_GL,ManagedElement=BB_AC365_GL,Equipment=1,FieldReplaceableUnit=RRUS-9_B3,RfPort=B 2583249128</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>2026-09-23 16:15:14</t>
+          <t>2026-09-24 07:59:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-24 16:39:16
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,10 +424,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -518,17 +518,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC203</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SINFRA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-23 22:18:28</t>
+          <t>2026-09-24 08:25:13</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-23 22:18:28</t>
+          <t>2026-09-24 08:25:13</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=81/178, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,39 +578,39 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC464</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>OUELLE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-22 10:48:07</t>
+          <t>2026-09-24 13:10:55</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-22 10:48:07</t>
+          <t>2026-09-24 13:10:55</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,49 +635,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BEKOUKOUIFIN</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ET337</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BB_ET337_GL</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Critical Temperature Taken Out of Service</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-24 06:44:08</t>
+          <t>2026-09-24 13:48:54</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-24 07:54:42</t>
+          <t>2026-09-24 13:48:54</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET337_GL,ManagedElement=BB_ET337_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2576049599</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=92/198, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC186</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>MBAHIAKRO</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Board Temperature Unacceptable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-24 14:48:55</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-24 14:48:55</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=80/176, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>DABOU_SODECI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>AC932</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_AC932_W</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-24 10:18:02</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-24 10:18:02</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2583202212</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>DABOU_SODECI</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>AC932</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_AC932_W</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-24 13:37:18</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-24 13:37:18</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-2 2583195875</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,39 +913,39 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-24 15:10:27</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-24 15:10:27</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
@@ -1059,12 +1059,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,54 +1114,54 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC832</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BAONFLA</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>High Temp</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-23 23:55:14</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-23 23:55:14</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,34 +1171,34 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1208,12 +1208,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1248,24 +1248,24 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,54 +1382,54 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>ABOISSO_MUNICIPALITE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>ET545</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>Microwave</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>ET545-ML6691</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>High Temperature</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-24 15:02:27</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-24 15:02:27</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>SubNetwork=MINILINK,MeContext=ET545-ML6691,ManagedElement=ET545-ML6691,NPU_1003=1/4 2582421010</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,39 +1449,39 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>TERMINAL_2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>ET903</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>BB_ET903_WL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
+          <t>Indoor RAP Temperature Exceptional</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-24 15:58:18</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-24 15:58:18</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET903_WL,ManagedElement=BB_ET903_WL,Equipment=1,FieldReplaceableUnit=RD-1-3 2576221744</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,24 +1516,24 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,57 +1583,54 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>250</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-12 09:15:07</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1643,53 +1640,50 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>20</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1698,12 +1692,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1713,67 +1707,64 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1783,67 +1774,64 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>31</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1853,67 +1841,64 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>245</v>
+          <t>RF Reflected Power High</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1923,17 +1908,17 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
@@ -1945,12 +1930,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1960,7 +1945,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1978,12 +1963,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-23 20:55:54</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-23 20:55:54</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1993,7 +1978,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=351, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2003,40 +1988,43 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>WAC183</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>RfPortReflectedPowerTooHigh</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>31</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2045,12 +2033,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:26</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-10 14:12:06</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2060,50 +2048,53 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>OKROMODOU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AC791</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WAC791</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>31</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2112,12 +2103,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:43</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2127,50 +2118,53 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DOUGODOU</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET197</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>WET197</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>245</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2179,12 +2173,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-19 09:34:45</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2194,64 +2188,67 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BLAHOU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC788</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WAC788</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>250</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-24 13:49:46</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-19 09:37:11</t>
+          <t>2026-09-24 13:49:46</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2261,64 +2258,67 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>WAC534</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>20</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-31 11:22:58</t>
+          <t>2026-09-24 14:33:55</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-31 12:14:01</t>
+          <t>2026-09-24 14:33:55</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2328,64 +2328,67 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BONDOUKOU</t>
+          <t>ZEGA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AC182</t>
+          <t>ET861</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>WAC182</t>
+          <t>ZEGA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>20</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-24 04:28:23</t>
+          <t>2026-09-24 15:33:43</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-24 04:28:23</t>
+          <t>2026-09-24 15:33:43</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2395,34 +2398,34 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC182,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583505337</t>
+          <t>Cabinet No.=0, Subrack No.=91, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=375, RF Port=NULL</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2432,12 +2435,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>RfPortReflectedPowerTooHigh</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2447,12 +2450,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-24 06:21:35</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-24 07:18:57</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2462,7 +2465,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2472,7 +2475,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
@@ -2484,22 +2487,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>OKROMODOU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC791</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>WAC791</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2514,12 +2517,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-24 06:30:28</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-24 07:21:57</t>
+          <t>2026-08-19 09:34:43</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2529,7 +2532,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576000533</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC791,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564611251</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2539,24 +2542,24 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>KAMAGAYA</t>
+          <t>DOUGODOU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AC731</t>
+          <t>ET197</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2566,7 +2569,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WAC731</t>
+          <t>WET197</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2581,12 +2584,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-24 07:36:55</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-24 07:36:55</t>
+          <t>2026-08-19 09:34:45</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2596,7 +2599,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC731,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583487709</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET197,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564635969</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2606,7 +2609,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
@@ -2618,12 +2621,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>BLAHOU</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC788</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2633,7 +2636,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>WAC788</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2648,12 +2651,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-24 07:40:17</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-24 07:40:17</t>
+          <t>2026-08-19 09:37:11</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2663,7 +2666,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133866</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC788,ManagedElement=1,TransportNetwork=1,Synchronization=1 2564625068</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2673,24 +2676,24 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>BOUBOURY</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC534</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2700,7 +2703,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WAC781</t>
+          <t>WAC534</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2715,12 +2718,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-24 07:41:29</t>
+          <t>2026-08-31 11:22:58</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-24 07:41:29</t>
+          <t>2026-08-31 12:14:01</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2730,7 +2733,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576133857</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC534,ManagedElement=1,TransportNetwork=1,Synchronization=1 2571911293</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2740,34 +2743,34 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KROKROM</t>
+          <t>ADIAPOTO</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AC221</t>
+          <t>ET493</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>WAC221</t>
+          <t>LET493</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2782,12 +2785,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:13</t>
+          <t>2026-09-24 10:35:41</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:13</t>
+          <t>2026-09-24 10:35:41</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2797,7 +2800,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC221,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582833603</t>
+          <t>SubNetwork=EnodeB,MeContext=LET493,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583563415</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2807,7 +2810,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2822,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DAKPADOU</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AC767</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2834,7 +2837,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WAC767</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2849,12 +2852,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:14</t>
+          <t>2026-09-24 15:51:27</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:14</t>
+          <t>2026-09-24 15:51:27</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2864,7 +2867,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC767,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576235471</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2575962292</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2874,7 +2877,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
@@ -2886,27 +2889,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SASSANDRA</t>
+          <t>SASSANDRA_PHARE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AC161</t>
+          <t>ET371</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>4G</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WAC161</t>
+          <t>LET371</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>TU Oscillator Temperature Fault</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2916,12 +2919,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:22</t>
+          <t>2026-09-24 15:58:52</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:22</t>
+          <t>2026-09-24 15:58:52</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2931,7 +2934,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WAC161,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583331220</t>
+          <t>SubNetwork=EnodeB,MeContext=LET371,ManagedElement=1,Equipment=1,Subrack=1,Slot=1,PlugInUnit=1,TimingUnit=1 2583669353</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2941,54 +2944,54 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NIAMBEZARIA</t>
+          <t>MARC_AKWABA2</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ET196</t>
+          <t>ET001</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>WET196</t>
+          <t>ET001-OSmon</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Temperature Outside Limits</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:24</t>
+          <t>1970-01-11 20:41:00</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:24</t>
+          <t>1970-01-11 20:41:00</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2998,7 +3001,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET196,ManagedElement=1,TransportNetwork=1,Synchronization=1 2580997386</t>
+          <t>SubNetwork=TCU,MeContext=ET001-OSmon,STN=0,Equipment=0 2583632594</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3008,54 +3011,54 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KOTCHERI</t>
+          <t>EBOINDA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ET151</t>
+          <t>ET149</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>WET151</t>
+          <t>ET149-OSmon</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Temperature is near limits</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:28</t>
+          <t>2007-02-08 15:23:26</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:28</t>
+          <t>2007-02-08 15:23:26</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3065,7 +3068,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_GROUP,MeContext=WET151,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576384110</t>
+          <t>SubNetwork=TCU,MeContext=ET149-OSmon,STN=0,Equipment=0 2583648606</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3075,54 +3078,57 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CANTONDOUGOU</t>
+          <t>GOUDI</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ET490</t>
+          <t>ET148</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>WET490</t>
+          <t>BB_ET148_GL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1.6</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:28</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:28</t>
+          <t>2026-06-17 12:12:52</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3132,7 +3138,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET490,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582774827</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3142,24 +3148,24 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CHIEPO</t>
+          <t>ADAOU</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ET141</t>
+          <t>AC548</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3169,27 +3175,30 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>WET141</t>
+          <t>BB_AC548_W</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>2.1</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:30</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:30</t>
+          <t>2026-08-19 15:48:55</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3199,7 +3208,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_GROUP,MeContext=WET141,ManagedElement=1,TransportNetwork=1,Synchronization=1 2576334017</t>
+          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3209,54 +3218,57 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>NONOUAN</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AC760</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>WAC760</t>
+          <t>BB_ET425_GL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1.7</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:34</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:34</t>
+          <t>2026-09-08 21:18:56</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3266,7 +3278,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582782842</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3276,54 +3288,57 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SASSANDRA_PHARE</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ET371</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>LET371</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1.7</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:43</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:43</t>
+          <t>2026-09-09 13:41:30</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3333,7 +3348,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LET371,ManagedElement=1,TransportNetwork=1,Synchronization=1 2582774837</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3343,54 +3358,57 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>NONOUAN</t>
+          <t>YOP_BAFOND</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>AC760</t>
+          <t>IM522</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>2G,3G</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>LAC760</t>
+          <t>BB_IM522_GW</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>4.6</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-09-24 07:48:07</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-09-24 07:48:07</t>
+          <t>2026-09-19 11:33:44</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3400,7 +3418,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC760,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583487821</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3410,54 +3428,57 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>NERO_PALMCI</t>
+          <t>SONGON_BEL_HORIZON</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ET214</t>
+          <t>ET815</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>WET214</t>
+          <t>BB_ET815_GL</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
-        </is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1.6</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-09-24 07:48:21</t>
+          <t>2026-09-22 09:23:21</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-09-24 07:48:21</t>
+          <t>2026-09-22 09:23:21</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3467,7 +3488,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET214,ManagedElement=1,TransportNetwork=1,Synchronization=1 2583505436</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3477,24 +3498,24 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>STAR_2</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC365</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3504,7 +3525,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>BB_AC365_GL</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3513,7 +3534,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>1.6</v>
+        <v>3.3</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -3522,12 +3543,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-23 14:42:02</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-06-17 12:12:52</t>
+          <t>2026-09-23 14:42:02</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3537,7 +3558,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2568857213</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC365_GL,ManagedElement=BB_AC365_GL,Equipment=1,FieldReplaceableUnit=RRUS-9_B3,RfPort=B 2583249128</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -3547,34 +3568,34 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ADAOU</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>AC548</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>BB_AC548_W</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3583,7 +3604,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>2.1</v>
+        <v>5</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -3592,12 +3613,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-24 12:55:37</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-08-19 15:48:55</t>
+          <t>2026-09-24 12:55:37</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3607,7 +3628,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC548_W,ManagedElement=BB_AC548_W,Equipment=1,FieldReplaceableUnit=RRU-2,RfPort=A 2568858592</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3617,34 +3638,34 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>KOUWEIT_PIERRE_GADIE</t>
+          <t>TRANSUA</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ET425</t>
+          <t>AC566</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>BB_ET425_GL</t>
+          <t>BB_AC566_W</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3653,7 +3674,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -3662,12 +3683,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-24 15:32:07</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-09-08 21:18:56</t>
+          <t>2026-09-24 15:32:07</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3677,7 +3698,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET425_GL,ManagedElement=BB_ET425_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B20,RfPort=A 2570618600</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3687,7 +3708,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>
@@ -3699,12 +3720,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>GESCO</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC314</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3714,7 +3735,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>BB_AC314_GL</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3723,7 +3744,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1.7</v>
+        <v>4.1</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3732,12 +3753,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-24 15:35:22</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-09-09 13:41:30</t>
+          <t>2026-09-24 15:35:22</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3747,7 +3768,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2576931392</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=B 2581257421</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3757,427 +3778,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-09-24 07:59:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>GESCO</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>AC314</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>BB_AC314_GL</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>5</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-09-18 10:35:17</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:36:44</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC314_GL,ManagedElement=BB_AC314_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2581177027</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:59:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>YOP_BAFOND</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>IM522</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2G,3G</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>BB_IM522_GW</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:33:44</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2026-09-19 11:33:44</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC05,MeContext=BB_IM522_GW,ManagedElement=BB_IM522_GW,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2572742241</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:59:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>ABIDJAN 02</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>SONGON_BEL_HORIZON</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>ET815</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>BB_ET815_GL</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-09-22 09:23:21</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-09-22 09:23:21</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2582145144</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:59:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>ABENGOUROU</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>TRANSUA</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>AC566</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>3G</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>BB_AC566_W</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-09-23 03:35:57</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2026-09-23 03:35:57</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_AC566_W,ManagedElement=BB_AC566_W,Equipment=1,FieldReplaceableUnit=RRUS-5,RfPort=A 2573870704</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:59:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>ABIDJAN 03</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>STAR_2</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>AC365</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>BB_AC365_GL</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>2026-09-23 14:42:02</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>2026-09-23 14:42:02</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC365_GL,ManagedElement=BB_AC365_GL,Equipment=1,FieldReplaceableUnit=RRUS-9_B3,RfPort=B 2583249128</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:59:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ABIDJAN 04</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>YAKASSE_ME</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>AC543</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>2G,4G</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>BB_AC543_GL</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:04:03</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:04:03</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC543_GL,ManagedElement=BB_AC543_GL,Equipment=1,FieldReplaceableUnit=RRUS-7_B1B3,RfPort=D 2583350904</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>ERICSSON</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>2026-09-24 07:59:55</t>
+          <t>2026-09-24 16:18:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour automatique 2026-09-25 00:33:14
</commit_message>
<xml_diff>
--- a/suivi_vswr.xlsx
+++ b/suivi_vswr.xlsx
@@ -424,10 +424,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N49"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -438,7 +438,7 @@
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="204" customWidth="1" min="12" max="12"/>
+    <col width="208" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
@@ -523,12 +523,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>AC501</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BEDIALA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-24 08:25:13</t>
+          <t>2026-09-24 16:04:21</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-24 08:25:13</t>
+          <t>2026-09-24 16:04:21</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -578,34 +578,34 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AC464</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OUELLE</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-24 13:10:55</t>
+          <t>2026-09-24 18:43:39</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-24 13:10:55</t>
+          <t>2026-09-24 18:43:39</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=90/194, Specific Problem=Temperature too High</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=5, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -645,39 +645,39 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>NDAKRO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AC501</t>
+          <t>ET471</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BEDIALA</t>
+          <t>BB_ET471_W</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-24 13:48:54</t>
+          <t>2026-09-24 18:53:06</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-24 13:48:54</t>
+          <t>2026-09-24 18:53:06</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -702,49 +702,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=7, Board Type=UMPT, Current Board Temperature (C/F)=92/198, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>BOUNA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AC186</t>
+          <t>AC288</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>MBAHIAKRO</t>
+          <t>BB_AC288_GL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-24 14:48:55</t>
+          <t>2026-09-24 23:26:09</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-24 14:48:55</t>
+          <t>2026-09-24 23:26:09</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -769,49 +769,49 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=16, Board Type=FAN, Current Board Temperature (C/F)=80/176, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC288_GL,ManagedElement=BB_AC288_GL,Equipment=1,FieldReplaceableUnit=RRU-5 2583790366</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DABOU_SODECI</t>
+          <t>NIAPIDOU</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AC932</t>
+          <t>AC816</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BB_AC932_W</t>
+          <t>BB_AC816_GL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-24 10:18:02</t>
+          <t>2026-08-13 15:59:47</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-24 10:18:02</t>
+          <t>2026-09-09 12:51:17</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-3 2583202212</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DABOU_SODECI</t>
+          <t>UIBA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC932</t>
+          <t>ET323</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BB_AC932_W</t>
+          <t>BB_ET323_GL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-24 13:37:18</t>
+          <t>2026-08-22 15:10:02</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-24 13:37:18</t>
+          <t>2026-09-09 13:00:42</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC932_W,ManagedElement=BB_AC932_W,Equipment=1,FieldReplaceableUnit=PSU-2 2583195875</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -913,39 +913,39 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NDAKRO</t>
+          <t>AVOCATIER</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ET471</t>
+          <t>AC376</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BB_ET471_W</t>
+          <t>BB_AC376_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Current Too High</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-24 15:10:27</t>
+          <t>2026-09-08 11:53:38</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-24 15:10:27</t>
+          <t>2026-09-18 00:43:34</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_ET471_W,ManagedElement=BB_ET471_W,Equipment=1,FieldReplaceableUnit=PSU-1 2575637619</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -980,24 +980,24 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NIAPIDOU</t>
+          <t>PHANIE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AC816</t>
+          <t>AC403</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_AC816_GL</t>
+          <t>BB_AC403_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-13 15:59:47</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09 12:51:17</t>
+          <t>2026-09-09 12:47:16</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC816_GL,ManagedElement=BB_AC816_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2568853337</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
@@ -1059,12 +1059,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UIBA</t>
+          <t>ZOO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ET323</t>
+          <t>ET076</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_ET323_GL</t>
+          <t>BB_ET076_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-22 15:10:02</t>
+          <t>2026-09-10 12:30:37</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09 13:00:42</t>
+          <t>2026-09-15 14:56:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET323_GL,ManagedElement=BB_ET323_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=R 2568868793</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1114,24 +1114,24 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AVOCATIER</t>
+          <t>ATTOBAN_ST_BERNARD</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AC376</t>
+          <t>ET408</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BB_AC376_GL</t>
+          <t>BB_ET408_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-08 11:53:38</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-18 00:43:34</t>
+          <t>2026-09-22 14:08:18</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC376_GL,ManagedElement=BB_AC376_GL,Equipment=1,FieldReplaceableUnit=RRU-7,RfPort=R 2573978535</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1181,54 +1181,54 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PHANIE</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AC403</t>
+          <t>AC832</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BB_AC403_GL</t>
+          <t>BAONFLA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>High Temp</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-24 21:17:36</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-09 12:47:16</t>
+          <t>2026-09-24 21:17:36</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1238,34 +1238,34 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC403_GL,ManagedElement=BB_AC403_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2568853345</t>
+          <t>Cabinet No.=0, Subrack No.=0, Slot No.=19, Port No.=3, Board Type=UPEU, Manager Cabinet No.=NULL, Manager Subrack No.=NULL, User Label=NULL</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ZOO</t>
+          <t>JERUSALEM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ET076</t>
+          <t>AC033</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_ET076_GL</t>
+          <t>BB_AC033_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-10 12:30:37</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-15 14:56:00</t>
+          <t>2026-07-19 17:01:06</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET076_GL,ManagedElement=BB_ET076_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=R 2576575822</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ATTOBAN_ST_BERNARD</t>
+          <t>JACQUEVIL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ET408</t>
+          <t>AC211</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_ET408_GL</t>
+          <t>BB_AC211_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Current Too High</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-22 14:08:18</t>
+          <t>2026-07-24 00:30:05</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET408_GL,ManagedElement=BB_ET408_GL,Equipment=1,FieldReplaceableUnit=RRU-8,RfPort=R 2582808868</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1382,54 +1382,54 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ABOISSO_MUNICIPALITE</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ET545</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Microwave</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ET545-ML6691</t>
+          <t>BB_AC183_GL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>High Temperature</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-24 15:02:27</t>
+          <t>2026-07-29 00:48:36</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-24 15:02:27</t>
+          <t>2026-09-10 14:07:38</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>SubNetwork=MINILINK,MeContext=ET545-ML6691,ManagedElement=ET545-ML6691,NPU_1003=1/4 2582421010</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1449,39 +1449,39 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TERMINAL_2</t>
+          <t>NOUVEAU_QUARTIER</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ET903</t>
+          <t>AC710</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_ET903_WL</t>
+          <t>BB_AC710_GL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Indoor RAP Temperature Exceptional</t>
+          <t>RF Reflected Power High</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-24 15:58:18</t>
+          <t>2026-09-02 02:49:52</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-24 15:58:18</t>
+          <t>2026-09-20 02:39:57</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET903_WL,ManagedElement=BB_ET903_WL,Equipment=1,FieldReplaceableUnit=RD-1-3 2576221744</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>JERUSALEM</t>
+          <t>KOWEIT</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AC033</t>
+          <t>AC624</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_AC033_GL</t>
+          <t>BB_AC624_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-19 17:01:06</t>
+          <t>2026-09-03 19:22:43</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC033_GL,ManagedElement=BB_AC033_GL,Equipment=1,FieldReplaceableUnit=RRUS-2_B20,RfPort=A 2568853780</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1583,24 +1583,24 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>JACQUEVIL</t>
+          <t>STBENOIT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AC211</t>
+          <t>AC400</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_AC211_GL</t>
+          <t>BB_AC400_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-10 16:09:55</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-07-24 00:30:05</t>
+          <t>2026-09-20 22:33:02</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC211_GL,ManagedElement=BB_AC211_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B20,RfPort=A 2568858383</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1650,40 +1650,43 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DJIMINISSO</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AC183</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BB_AC183_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>20</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1692,12 +1695,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-07-29 00:48:36</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-10 14:07:38</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1707,64 +1710,67 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC183_GL,ManagedElement=BB_AC183_GL,Equipment=1,FieldReplaceableUnit=RRU-12_B8,RfPort=A 2568862207</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NOUVEAU_QUARTIER</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AC710</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BB_AC710_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>31</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-02 02:49:52</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-20 02:39:57</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1774,64 +1780,67 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC710_GL,ManagedElement=BB_AC710_GL,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2572946238</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KOWEIT</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AC624</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BB_AC624_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>31</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-03 19:22:43</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1841,64 +1850,67 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC624_GL,ManagedElement=BB_AC624_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=A 2574100444</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>STBENOIT</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AC400</t>
+          <t>ET924</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BB_AC400_GL</t>
+          <t>YEPLEU</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RF Reflected Power High</t>
-        </is>
+          <t>RF Unit VSWR Threshold Crossed</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>245</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-10 16:09:55</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-20 22:33:02</t>
+          <t>2026-09-21 08:27:43</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1908,34 +1920,34 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC400_GL,ManagedElement=BB_AC400_GL,Equipment=1,FieldReplaceableUnit=RRU-9,RfPort=B 2574042620</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC449</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1945,7 +1957,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BUYO</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1954,7 +1966,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1963,12 +1975,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-24 13:49:46</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-24 13:49:46</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1978,7 +1990,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=415, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1988,7 +2000,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
@@ -2000,12 +2012,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET673</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2015,7 +2027,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BANNEU</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2024,21 +2036,21 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-24 22:59:55</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-24 22:59:55</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2048,7 +2060,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=2, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=350, RF Port=NULL</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2058,43 +2070,40 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>DJIMINISSO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>AC183</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>WAC183</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>31</v>
+          <t>RfPortReflectedPowerTooHigh</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2103,12 +2112,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-07-29 00:48:26</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-10 14:12:06</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2118,67 +2127,64 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=31, Output Power (0.1 dBm)=369, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC183,ManagedElement=1,Equipment=1,RbsSubrack=1,RbsSlot=9,AuxPlugInUnit=RUW-1,DeviceGroup=RUW,AiDeviceSet=1,AiDevice=1 2568851532</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>GRAND_JACQUES</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ET924</t>
+          <t>ET489</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>YEPLEU</t>
+          <t>BB_ET489_W</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>245</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-24 17:24:07</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-21 08:27:43</t>
+          <t>2026-09-24 17:24:07</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2188,67 +2194,64 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=0, Board Type=MRRU, VSWR Alarm Threshold (0.1)=30, VSWR(0.1)=245, Output Power (0.1 dBm)=352, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_ET489_W,ManagedElement=BB_ET489_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2583687566</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>GRAND_JACQUES</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AC449</t>
+          <t>ET489</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BUYO</t>
+          <t>BB_ET489_W</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>250</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-24 13:49:46</t>
+          <t>2026-09-24 17:24:07</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-24 13:49:46</t>
+          <t>2026-09-24 17:24:07</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2258,67 +2261,64 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=92, Slot No.=0, TX Channel No.=1, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=250, Output Power (0.1 dBm)=370, RF Port=NULL</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_ET489_W,ManagedElement=BB_ET489_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2583687567</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>GRAND_JACQUES</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ET673</t>
+          <t>ET489</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BANNEU</t>
+          <t>BB_ET489_GL</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>RF Unit VSWR Threshold Crossed</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>20</v>
+          <t>Sync Frequency Reference Not Reliable</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-24 14:33:55</t>
+          <t>2026-09-24 17:24:09</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-24 14:33:55</t>
+          <t>2026-09-24 17:24:09</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2328,67 +2328,64 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=90, Slot No.=0, TX Channel No.=3, Board Type=MRRU, VSWR Alarm Threshold (0.1)=20, VSWR(0.1)=20, Output Power (0.1 dBm)=354, RF Port=NULL</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET489_GL,ManagedElement=BB_ET489_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2583687577</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-24 16:18:41</t>
+          <t>2026-09-25 00:18:05</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="i